<commit_message>
Added logic to store matches on device
</commit_message>
<xml_diff>
--- a/DERT_Scouting_REBUILT.xlsx
+++ b/DERT_Scouting_REBUILT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JD Projects\DERT\QRCodeTest\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JD Projects\DERT\Scoutning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF397B7B-D469-44DA-93AF-864F4F16430E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1A728EB-0E8A-4A7F-AD60-C3C41C494743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6400" yWindow="4110" windowWidth="19200" windowHeight="11170" xr2:uid="{22C98769-AA28-4D3C-9C55-FAEF3A66851A}"/>
+    <workbookView xWindow="31920" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{10593C7C-49B4-48F1-828D-C303B4AFBAA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="132">
+  <si>
+    <t>Schema</t>
+  </si>
   <si>
     <t>Match type</t>
   </si>
@@ -276,7 +279,7 @@
     <t>IMPORTING MATCHES</t>
   </si>
   <si>
-    <t>Go to the Scans sheet and click the first EMPTY cell in column A (Match type).</t>
+    <t>Go to the Scans sheet and click the first EMPTY cell in column A (Schema).</t>
   </si>
   <si>
     <t>Scan the student's QR code. The whole match fills one row and the cursor moves to the next row automatically.</t>
@@ -318,16 +321,28 @@
     <t>Requires Microsoft 365 / Excel 2021 or newer (uses UNIQUE, SORTBY, FILTER, HSTACK).</t>
   </si>
   <si>
+    <t>Schema (column A) is filled in by every QR code (S39-44228b4d for this workbook). A RED row came from a different version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   of the scouting form, so its answers are in the wrong columns: delete it, update the app on that phone (open it on Wi-Fi), scan again.</t>
+  </si>
+  <si>
     <t>IF YOU CHANGE THE WEB FORM</t>
   </si>
   <si>
-    <t>Adding, removing or re-ordering fields in index.html changes the QR columns. Update the Scans headers to match</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   (the web app's QR screen has an 'Excel column headers' section you can copy), and check the Team Summary formulas.</t>
+    <t>Adding, removing or renaming fields in index.html changes the QR columns and the Schema stamp. Update the header list in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   build-excel.ps1 to match (the web app's QR screen has an 'Excel column headers' section you can copy) and rebuild this workbook,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   otherwise every new scan shows up red. Check the Team Summary formulas too.</t>
   </si>
   <si>
     <t>EXAMPLE ROW (what one scanned match looks like)</t>
+  </si>
+  <si>
+    <t>Schema:  S39-44228b4d</t>
   </si>
   <si>
     <t>Match type:  Qual</t>
@@ -606,7 +621,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -678,48 +703,49 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{434EB9A2-751B-49CA-A808-5C35DD6ACFC6}" name="Scans" displayName="Scans" ref="A1:AM2" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:AM2" xr:uid="{434EB9A2-751B-49CA-A808-5C35DD6ACFC6}"/>
-  <tableColumns count="39">
-    <tableColumn id="1" xr3:uid="{0C09BACE-88C4-4F6D-9A14-F6BAD29583B6}" name="Match type"/>
-    <tableColumn id="2" xr3:uid="{D3BEE4B7-9BD1-4657-AD49-D214AA2D0239}" name="Match #"/>
-    <tableColumn id="3" xr3:uid="{DE4F3FE4-6557-4CAE-890D-BBDDA3289B4D}" name="Team #"/>
-    <tableColumn id="4" xr3:uid="{846F38D0-0488-4BEB-92EF-A5751D75E21B}" name="Alliance"/>
-    <tableColumn id="5" xr3:uid="{839A7DC6-B5F1-41D4-B63F-CB8E529907D7}" name="Station"/>
-    <tableColumn id="6" xr3:uid="{F56EC7A0-DA20-4AFA-A37E-5D359A88464F}" name="Scout name"/>
-    <tableColumn id="7" xr3:uid="{31253C93-6EFE-42B6-B1AB-FAA93AA6FC8E}" name="Robot on field?"/>
-    <tableColumn id="8" xr3:uid="{F2C6CB14-7520-40D7-9633-B2676B137679}" name="Starting position"/>
-    <tableColumn id="9" xr3:uid="{2FED543A-E69A-43DF-9789-18EDF347A750}" name="Fuel preloaded"/>
-    <tableColumn id="10" xr3:uid="{A59B2E7B-60B9-4EE1-9BEC-CE850468CCF7}" name="Auto fuel scored"/>
-    <tableColumn id="11" xr3:uid="{0559686A-DFA3-465B-8E86-40B66ED113DB}" name="Auto fuel missed"/>
-    <tableColumn id="12" xr3:uid="{D1004C55-CA52-4290-B502-39C5437668BF}" name="Auto path"/>
-    <tableColumn id="13" xr3:uid="{DAA04B2B-629E-435A-B25B-120F45E5DA1C}" name="Picked up fuel from"/>
-    <tableColumn id="14" xr3:uid="{24E5E5C9-7DC3-452A-9AFE-C2266937BB7B}" name="Tower climb in auto"/>
-    <tableColumn id="15" xr3:uid="{829037BE-82CA-43C2-AB90-63CA5D011A11}" name="Teleop fuel scored"/>
-    <tableColumn id="16" xr3:uid="{1C93E913-9121-455D-8148-A9D8F0C24241}" name="Teleop fuel missed"/>
-    <tableColumn id="17" xr3:uid="{02C6E0D0-EA4C-4CD9-A8F9-EC69334575FA}" name="Intake from"/>
-    <tableColumn id="18" xr3:uid="{933BE325-87DF-46C1-AEB6-0B7B5B217A56}" name="Shoots from"/>
-    <tableColumn id="19" xr3:uid="{B8A9F833-3F35-4314-9B8F-0FA42AA7BD95}" name="Drives over / through"/>
-    <tableColumn id="20" xr3:uid="{D5A0CFE2-D6ED-45B4-A2BE-52887E888635}" name="Inactive Hub behavior"/>
-    <tableColumn id="21" xr3:uid="{1E8CA0DE-01A8-4C5E-A7C2-510D0C253D55}" name="Fuel it can carry"/>
-    <tableColumn id="22" xr3:uid="{A47DE0DA-46A5-4BDC-B95A-EE9167B21CE0}" name="Played defense"/>
-    <tableColumn id="23" xr3:uid="{C30D06F4-AEF4-4949-AC7B-B98A4BF0843B}" name="Was defended"/>
-    <tableColumn id="24" xr3:uid="{3B093ECD-186D-4667-898F-8D65DB4FA487}" name="Tower climb"/>
-    <tableColumn id="25" xr3:uid="{A6AFC528-421B-4717-9E53-D9B3DF570A1D}" name="Climb time"/>
-    <tableColumn id="26" xr3:uid="{01350470-19B4-4AEF-8CA4-581611FE6A43}" name="Driver skill"/>
-    <tableColumn id="27" xr3:uid="{71F0DFA4-B358-40E7-9207-3D58EBC79E63}" name="Robot speed"/>
-    <tableColumn id="28" xr3:uid="{3ED4F6D3-4C72-42ED-B840-257319034089}" name="Shooting accuracy"/>
-    <tableColumn id="29" xr3:uid="{F882D7F3-DCCA-47BD-9291-9B5904A1A882}" name="Problems"/>
-    <tableColumn id="30" xr3:uid="{076FE577-99CF-4067-8F86-9295ADA4C37E}" name="Minor fouls"/>
-    <tableColumn id="31" xr3:uid="{380F157F-B441-48C1-98F7-7297022DBCD5}" name="Major fouls"/>
-    <tableColumn id="32" xr3:uid="{A3425F11-D755-400E-A8B3-02D09CFF6E75}" name="Card"/>
-    <tableColumn id="33" xr3:uid="{D0643373-ED2A-4A16-9DB5-B4EF866DB248}" name="Pick?"/>
-    <tableColumn id="34" xr3:uid="{E0CB741D-2B61-4487-A882-AB7B6FAEB8CB}" name="Observations"/>
-    <tableColumn id="35" xr3:uid="{9775960A-2F1A-4A44-B568-34629D34970A}" name="Auto pts" dataDxfId="4"/>
-    <tableColumn id="36" xr3:uid="{F7A0FA6F-0FBF-4D97-8848-FAF52CA97FD0}" name="Teleop fuel pts" dataDxfId="3"/>
-    <tableColumn id="37" xr3:uid="{A514E2E6-FCBD-4518-905F-6B34BC86043E}" name="Climb pts" dataDxfId="2"/>
-    <tableColumn id="38" xr3:uid="{36B3D2B0-A685-44CD-81D8-80D3DE2430C2}" name="Total pts" dataDxfId="1"/>
-    <tableColumn id="39" xr3:uid="{09994039-F07C-460F-AA59-4EB8F521EC82}" name="Submitted"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CAED70B0-DE09-4E28-B128-B5A1BB44310D}" name="Scans" displayName="Scans" ref="A1:AN2" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:AN2" xr:uid="{CAED70B0-DE09-4E28-B128-B5A1BB44310D}"/>
+  <tableColumns count="40">
+    <tableColumn id="1" xr3:uid="{48E27B7A-CA15-4AF9-A6CD-59A104743BAE}" name="Schema"/>
+    <tableColumn id="2" xr3:uid="{3F74FAA0-76E7-481E-91CB-1C90A9CF2B12}" name="Match type"/>
+    <tableColumn id="3" xr3:uid="{C9F053CB-FB12-4D1F-8C93-08C560DFC0E2}" name="Match #"/>
+    <tableColumn id="4" xr3:uid="{06B6EA5A-F115-4773-9379-20F5C0DAF37E}" name="Team #"/>
+    <tableColumn id="5" xr3:uid="{3E24579D-CDA3-49E8-9A74-7BF769A48F1E}" name="Alliance"/>
+    <tableColumn id="6" xr3:uid="{EB7C3CC1-7DFA-45C5-AB39-148111D410E1}" name="Station"/>
+    <tableColumn id="7" xr3:uid="{E32A9544-CA6B-4E86-9F05-546479D69095}" name="Scout name"/>
+    <tableColumn id="8" xr3:uid="{1E58C162-CE0B-4FD6-BD96-20A49C9E9DE4}" name="Robot on field?"/>
+    <tableColumn id="9" xr3:uid="{2908C53C-7956-4073-9D62-C7AB067E3B54}" name="Starting position"/>
+    <tableColumn id="10" xr3:uid="{C34C70C8-2B6C-44A5-9C4C-735B07C2E39B}" name="Fuel preloaded"/>
+    <tableColumn id="11" xr3:uid="{FFE72816-F277-49FF-A7ED-3FDB1370AA46}" name="Auto fuel scored"/>
+    <tableColumn id="12" xr3:uid="{C9695201-E184-46D5-A3E4-005CE86111BC}" name="Auto fuel missed"/>
+    <tableColumn id="13" xr3:uid="{891E0D14-5B92-4640-B5B2-EC1101E54B13}" name="Auto path"/>
+    <tableColumn id="14" xr3:uid="{46BF066C-AE5C-49E4-B141-47E3BED53038}" name="Picked up fuel from"/>
+    <tableColumn id="15" xr3:uid="{1F9A4E4C-40B0-409F-AF73-B675BB648ED8}" name="Tower climb in auto"/>
+    <tableColumn id="16" xr3:uid="{1A49E944-89D4-4A47-B178-DC532E2D8307}" name="Teleop fuel scored"/>
+    <tableColumn id="17" xr3:uid="{256461DD-35C7-417D-B2EF-40D13A572371}" name="Teleop fuel missed"/>
+    <tableColumn id="18" xr3:uid="{44711B57-5166-455B-A898-EEB0382E2649}" name="Intake from"/>
+    <tableColumn id="19" xr3:uid="{1381B124-5E8E-4CF1-8C49-32CFB943468F}" name="Shoots from"/>
+    <tableColumn id="20" xr3:uid="{5B427C04-D937-4C69-962D-55CE6045F356}" name="Drives over / through"/>
+    <tableColumn id="21" xr3:uid="{D40A23FC-D353-4C4C-94DC-00046D6B1377}" name="Inactive Hub behavior"/>
+    <tableColumn id="22" xr3:uid="{595D8CA2-E094-41E7-A1FF-82AE6F0A2620}" name="Fuel it can carry"/>
+    <tableColumn id="23" xr3:uid="{98274B37-39F3-4791-953A-B64B87F8DA11}" name="Played defense"/>
+    <tableColumn id="24" xr3:uid="{E3CD61A2-31AA-40FE-B7C4-C7B661282D0E}" name="Was defended"/>
+    <tableColumn id="25" xr3:uid="{6952C9B9-5BA2-467A-909C-8F644128CDD0}" name="Tower climb"/>
+    <tableColumn id="26" xr3:uid="{962B4FA8-F9B6-495A-9C7F-73FCAC29AE87}" name="Climb time"/>
+    <tableColumn id="27" xr3:uid="{7ECC41F7-DCCF-4170-8F78-F19D3C62E6F1}" name="Driver skill"/>
+    <tableColumn id="28" xr3:uid="{0BE98F09-D94D-4C74-8290-56F0F564BE40}" name="Robot speed"/>
+    <tableColumn id="29" xr3:uid="{6E39DAC0-6ED5-43B4-9568-35CA6F375292}" name="Shooting accuracy"/>
+    <tableColumn id="30" xr3:uid="{A28B5CA3-A61C-4C51-9AD7-9CB91A3CB0EA}" name="Problems"/>
+    <tableColumn id="31" xr3:uid="{93C242A1-A76B-4E0D-9A55-8E1467FD133A}" name="Minor fouls"/>
+    <tableColumn id="32" xr3:uid="{0B8104B6-C30D-4FF6-8919-20D9782D34C4}" name="Major fouls"/>
+    <tableColumn id="33" xr3:uid="{FD787B85-141E-4516-8AF5-DE66DD9320C0}" name="Card"/>
+    <tableColumn id="34" xr3:uid="{94017362-8D5A-4B97-8867-2490CB641F73}" name="Pick?"/>
+    <tableColumn id="35" xr3:uid="{6FBD70BA-77D9-4D54-809D-CA203835F4D5}" name="Observations"/>
+    <tableColumn id="36" xr3:uid="{23C8A014-2BDC-40A1-909F-FCC1B1571FC4}" name="Auto pts" dataDxfId="5"/>
+    <tableColumn id="37" xr3:uid="{C04EAA6B-2FD9-4C42-83DF-2AD7999B830C}" name="Teleop fuel pts" dataDxfId="4"/>
+    <tableColumn id="38" xr3:uid="{C35F15C7-C25F-495D-A2CE-3BAF28DA7465}" name="Climb pts" dataDxfId="3"/>
+    <tableColumn id="39" xr3:uid="{47944D55-9A84-4F6F-8C4D-58D13774EB23}" name="Total pts" dataDxfId="2"/>
+    <tableColumn id="40" xr3:uid="{B343C979-E0B1-4588-A630-713C73AC0F6C}" name="Submitted"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1041,17 +1067,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E06F1927-1439-4FD9-B08B-4053E97C7086}">
-  <dimension ref="A1:J71"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0794377D-845E-422E-B584-2063023B892B}">
+  <dimension ref="A1:J75"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.6328125" customWidth="1"/>
-    <col min="2" max="2" width="110.6328125" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="2" width="110.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1063,9 +1089,9 @@
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
     </row>
-    <row r="2" spans="1:10" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1077,361 +1103,386 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="5" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="13">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="13"/>
       <c r="B7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="13">
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="13">
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="13">
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="13">
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="13">
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="13">
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="13" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
-        <v>75</v>
-      </c>
       <c r="B19" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="18" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="B29" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B27" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="13"/>
-      <c r="B30" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="13"/>
+      <c r="B28" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="18" t="s">
+    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="18" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B33" s="19" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B34" s="19" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="13"/>
+      <c r="B32" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B35" s="19" t="s">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="13"/>
+      <c r="B33" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B36" s="19" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B37" s="19" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B38" s="19" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B39" s="19" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B40" s="19" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B41" s="19" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B42" s="19" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B43" s="19" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B44" s="19" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B45" s="19" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B46" s="19" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B47" s="19" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B48" s="19" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B49" s="19" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B50" s="19" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B51" s="19" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B52" s="19" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B53" s="19" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B54" s="19" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B55" s="19" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B56" s="19" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B57" s="19" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B58" s="19" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B59" s="19" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B60" s="19" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B61" s="19" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B62" s="19" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B63" s="19" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B64" s="19" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B65" s="19" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B66" s="19" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B67" s="19" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B68" s="19" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B69" s="19" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B70" s="19" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B71" s="19" t="s">
-        <v>126</v>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B72" s="19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B73" s="19" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B74" s="19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B75" s="19" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -1440,31 +1491,32 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10243D0D-A533-4842-9301-948849D0A4B4}">
-  <dimension ref="A1:AM1"/>
-  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7748A9FA-E3CB-4775-A77C-0AB17B65355F}">
+  <dimension ref="A1:AN1"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="5" width="10.6328125" customWidth="1"/>
-    <col min="6" max="6" width="14.6328125" customWidth="1"/>
-    <col min="7" max="7" width="10.6328125" customWidth="1"/>
-    <col min="8" max="8" width="11.6328125" customWidth="1"/>
-    <col min="9" max="11" width="10.6328125" customWidth="1"/>
-    <col min="12" max="12" width="30.6328125" customWidth="1"/>
-    <col min="13" max="13" width="22.6328125" customWidth="1"/>
-    <col min="14" max="16" width="10.6328125" customWidth="1"/>
-    <col min="17" max="17" width="30.6328125" customWidth="1"/>
-    <col min="18" max="18" width="26.6328125" customWidth="1"/>
-    <col min="19" max="19" width="14.6328125" customWidth="1"/>
-    <col min="20" max="20" width="30.6328125" customWidth="1"/>
-    <col min="21" max="28" width="10.6328125" customWidth="1"/>
-    <col min="29" max="29" width="24.6328125" customWidth="1"/>
-    <col min="30" max="33" width="10.6328125" customWidth="1"/>
-    <col min="34" max="34" width="50.6328125" customWidth="1"/>
-    <col min="35" max="38" width="10.6328125" style="4" customWidth="1"/>
-    <col min="39" max="39" width="20.6328125" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="12" width="10.7109375" customWidth="1"/>
+    <col min="13" max="13" width="30.7109375" customWidth="1"/>
+    <col min="14" max="14" width="22.7109375" customWidth="1"/>
+    <col min="15" max="17" width="10.7109375" customWidth="1"/>
+    <col min="18" max="18" width="30.7109375" customWidth="1"/>
+    <col min="19" max="19" width="26.7109375" customWidth="1"/>
+    <col min="20" max="20" width="14.7109375" customWidth="1"/>
+    <col min="21" max="21" width="30.7109375" customWidth="1"/>
+    <col min="22" max="29" width="10.7109375" customWidth="1"/>
+    <col min="30" max="30" width="24.7109375" customWidth="1"/>
+    <col min="31" max="34" width="10.7109375" customWidth="1"/>
+    <col min="35" max="35" width="50.7109375" customWidth="1"/>
+    <col min="36" max="39" width="10.7109375" style="4" customWidth="1"/>
+    <col min="40" max="40" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:40" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1582,8 +1634,16 @@
       <c r="AM1" s="3" t="s">
         <v>38</v>
       </c>
+      <c r="AN1" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:AN5000">
+    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
+      <formula>($A2&lt;&gt;"")*($A2&lt;&gt;"S39-44228b4d")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1592,18 +1652,18 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BEDA31-ABC4-4299-A9B3-ED1395476863}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B090277A-8788-44C6-A687-09498AEBA7FD}">
   <dimension ref="A1:AC304"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="18" width="11.6328125" customWidth="1"/>
-    <col min="19" max="19" width="3.6328125" customWidth="1"/>
-    <col min="20" max="29" width="11.6328125" customWidth="1"/>
+    <col min="1" max="18" width="11.7109375" customWidth="1"/>
+    <col min="19" max="19" width="3.7109375" customWidth="1"/>
+    <col min="20" max="29" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:29" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1623,9 +1683,9 @@
       <c r="Q1" s="5"/>
       <c r="R1" s="5"/>
     </row>
-    <row r="2" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1645,98 +1705,98 @@
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
     </row>
-    <row r="3" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="T3" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="R4" s="7" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="4" spans="1:29" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="T4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="W4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="X4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="Y4" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I4" s="7" t="s">
+      <c r="Z4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AA4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="O4" s="7" t="s">
+      <c r="AB4" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="P4" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q4" s="7" t="s">
+      <c r="AC4" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="R4" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="T4" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="U4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="V4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="W4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="X4" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="Y4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z4" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="AA4" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="AB4" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC4" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="str" cm="1">
         <f t="array" ref="A5">IFERROR(_xlfn._xlws.SORT(_xlfn.UNIQUE(_xlfn._xlws.FILTER(Scans[Team '#],Scans[Team '#]&lt;&gt;""))),"")</f>
         <v/>
@@ -1826,7 +1886,7 @@
       <c r="AB5" s="13"/>
       <c r="AC5" s="13"/>
     </row>
-    <row r="6" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6" s="8"/>
       <c r="B6" s="9"/>
       <c r="C6" s="10"/>
@@ -1856,7 +1916,7 @@
       <c r="AB6" s="13"/>
       <c r="AC6" s="13"/>
     </row>
-    <row r="7" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7" s="8"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10"/>
@@ -1886,7 +1946,7 @@
       <c r="AB7" s="13"/>
       <c r="AC7" s="13"/>
     </row>
-    <row r="8" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8" s="8"/>
       <c r="B8" s="9"/>
       <c r="C8" s="10"/>
@@ -1916,7 +1976,7 @@
       <c r="AB8" s="13"/>
       <c r="AC8" s="13"/>
     </row>
-    <row r="9" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10"/>
@@ -1946,7 +2006,7 @@
       <c r="AB9" s="13"/>
       <c r="AC9" s="13"/>
     </row>
-    <row r="10" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="8"/>
       <c r="B10" s="9"/>
       <c r="C10" s="10"/>
@@ -1976,7 +2036,7 @@
       <c r="AB10" s="13"/>
       <c r="AC10" s="13"/>
     </row>
-    <row r="11" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11" s="8"/>
       <c r="B11" s="9"/>
       <c r="C11" s="10"/>
@@ -2006,7 +2066,7 @@
       <c r="AB11" s="13"/>
       <c r="AC11" s="13"/>
     </row>
-    <row r="12" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
       <c r="B12" s="9"/>
       <c r="C12" s="10"/>
@@ -2036,7 +2096,7 @@
       <c r="AB12" s="13"/>
       <c r="AC12" s="13"/>
     </row>
-    <row r="13" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13" s="8"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10"/>
@@ -2066,7 +2126,7 @@
       <c r="AB13" s="13"/>
       <c r="AC13" s="13"/>
     </row>
-    <row r="14" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14" s="8"/>
       <c r="B14" s="9"/>
       <c r="C14" s="10"/>
@@ -2096,7 +2156,7 @@
       <c r="AB14" s="13"/>
       <c r="AC14" s="13"/>
     </row>
-    <row r="15" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15" s="8"/>
       <c r="B15" s="9"/>
       <c r="C15" s="10"/>
@@ -2126,7 +2186,7 @@
       <c r="AB15" s="13"/>
       <c r="AC15" s="13"/>
     </row>
-    <row r="16" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16" s="8"/>
       <c r="B16" s="9"/>
       <c r="C16" s="10"/>
@@ -2156,7 +2216,7 @@
       <c r="AB16" s="13"/>
       <c r="AC16" s="13"/>
     </row>
-    <row r="17" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
       <c r="B17" s="9"/>
       <c r="C17" s="10"/>
@@ -2186,7 +2246,7 @@
       <c r="AB17" s="13"/>
       <c r="AC17" s="13"/>
     </row>
-    <row r="18" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A18" s="8"/>
       <c r="B18" s="9"/>
       <c r="C18" s="10"/>
@@ -2216,7 +2276,7 @@
       <c r="AB18" s="13"/>
       <c r="AC18" s="13"/>
     </row>
-    <row r="19" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
       <c r="B19" s="9"/>
       <c r="C19" s="10"/>
@@ -2246,7 +2306,7 @@
       <c r="AB19" s="13"/>
       <c r="AC19" s="13"/>
     </row>
-    <row r="20" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="B20" s="9"/>
       <c r="C20" s="10"/>
@@ -2276,7 +2336,7 @@
       <c r="AB20" s="13"/>
       <c r="AC20" s="13"/>
     </row>
-    <row r="21" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
       <c r="B21" s="9"/>
       <c r="C21" s="10"/>
@@ -2306,7 +2366,7 @@
       <c r="AB21" s="13"/>
       <c r="AC21" s="13"/>
     </row>
-    <row r="22" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A22" s="8"/>
       <c r="B22" s="9"/>
       <c r="C22" s="10"/>
@@ -2336,7 +2396,7 @@
       <c r="AB22" s="13"/>
       <c r="AC22" s="13"/>
     </row>
-    <row r="23" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A23" s="8"/>
       <c r="B23" s="9"/>
       <c r="C23" s="10"/>
@@ -2366,7 +2426,7 @@
       <c r="AB23" s="13"/>
       <c r="AC23" s="13"/>
     </row>
-    <row r="24" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A24" s="8"/>
       <c r="B24" s="9"/>
       <c r="C24" s="10"/>
@@ -2396,7 +2456,7 @@
       <c r="AB24" s="13"/>
       <c r="AC24" s="13"/>
     </row>
-    <row r="25" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A25" s="8"/>
       <c r="B25" s="9"/>
       <c r="C25" s="10"/>
@@ -2426,7 +2486,7 @@
       <c r="AB25" s="13"/>
       <c r="AC25" s="13"/>
     </row>
-    <row r="26" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A26" s="8"/>
       <c r="B26" s="9"/>
       <c r="C26" s="10"/>
@@ -2456,7 +2516,7 @@
       <c r="AB26" s="13"/>
       <c r="AC26" s="13"/>
     </row>
-    <row r="27" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A27" s="8"/>
       <c r="B27" s="9"/>
       <c r="C27" s="10"/>
@@ -2486,7 +2546,7 @@
       <c r="AB27" s="13"/>
       <c r="AC27" s="13"/>
     </row>
-    <row r="28" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A28" s="8"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10"/>
@@ -2516,7 +2576,7 @@
       <c r="AB28" s="13"/>
       <c r="AC28" s="13"/>
     </row>
-    <row r="29" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A29" s="8"/>
       <c r="B29" s="9"/>
       <c r="C29" s="10"/>
@@ -2546,7 +2606,7 @@
       <c r="AB29" s="13"/>
       <c r="AC29" s="13"/>
     </row>
-    <row r="30" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A30" s="8"/>
       <c r="B30" s="9"/>
       <c r="C30" s="10"/>
@@ -2576,7 +2636,7 @@
       <c r="AB30" s="13"/>
       <c r="AC30" s="13"/>
     </row>
-    <row r="31" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A31" s="8"/>
       <c r="B31" s="9"/>
       <c r="C31" s="10"/>
@@ -2606,7 +2666,7 @@
       <c r="AB31" s="13"/>
       <c r="AC31" s="13"/>
     </row>
-    <row r="32" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A32" s="8"/>
       <c r="B32" s="9"/>
       <c r="C32" s="10"/>
@@ -2636,7 +2696,7 @@
       <c r="AB32" s="13"/>
       <c r="AC32" s="13"/>
     </row>
-    <row r="33" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A33" s="8"/>
       <c r="B33" s="9"/>
       <c r="C33" s="10"/>
@@ -2666,7 +2726,7 @@
       <c r="AB33" s="13"/>
       <c r="AC33" s="13"/>
     </row>
-    <row r="34" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A34" s="8"/>
       <c r="B34" s="9"/>
       <c r="C34" s="10"/>
@@ -2696,7 +2756,7 @@
       <c r="AB34" s="13"/>
       <c r="AC34" s="13"/>
     </row>
-    <row r="35" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A35" s="8"/>
       <c r="B35" s="9"/>
       <c r="C35" s="10"/>
@@ -2726,7 +2786,7 @@
       <c r="AB35" s="13"/>
       <c r="AC35" s="13"/>
     </row>
-    <row r="36" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A36" s="8"/>
       <c r="B36" s="9"/>
       <c r="C36" s="10"/>
@@ -2756,7 +2816,7 @@
       <c r="AB36" s="13"/>
       <c r="AC36" s="13"/>
     </row>
-    <row r="37" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A37" s="8"/>
       <c r="B37" s="9"/>
       <c r="C37" s="10"/>
@@ -2786,7 +2846,7 @@
       <c r="AB37" s="13"/>
       <c r="AC37" s="13"/>
     </row>
-    <row r="38" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A38" s="8"/>
       <c r="B38" s="9"/>
       <c r="C38" s="10"/>
@@ -2816,7 +2876,7 @@
       <c r="AB38" s="13"/>
       <c r="AC38" s="13"/>
     </row>
-    <row r="39" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A39" s="8"/>
       <c r="B39" s="9"/>
       <c r="C39" s="10"/>
@@ -2846,7 +2906,7 @@
       <c r="AB39" s="13"/>
       <c r="AC39" s="13"/>
     </row>
-    <row r="40" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A40" s="8"/>
       <c r="B40" s="9"/>
       <c r="C40" s="10"/>
@@ -2876,7 +2936,7 @@
       <c r="AB40" s="13"/>
       <c r="AC40" s="13"/>
     </row>
-    <row r="41" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A41" s="8"/>
       <c r="B41" s="9"/>
       <c r="C41" s="10"/>
@@ -2906,7 +2966,7 @@
       <c r="AB41" s="13"/>
       <c r="AC41" s="13"/>
     </row>
-    <row r="42" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A42" s="8"/>
       <c r="B42" s="9"/>
       <c r="C42" s="10"/>
@@ -2936,7 +2996,7 @@
       <c r="AB42" s="13"/>
       <c r="AC42" s="13"/>
     </row>
-    <row r="43" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A43" s="8"/>
       <c r="B43" s="9"/>
       <c r="C43" s="10"/>
@@ -2966,7 +3026,7 @@
       <c r="AB43" s="13"/>
       <c r="AC43" s="13"/>
     </row>
-    <row r="44" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A44" s="8"/>
       <c r="B44" s="9"/>
       <c r="C44" s="10"/>
@@ -2996,7 +3056,7 @@
       <c r="AB44" s="13"/>
       <c r="AC44" s="13"/>
     </row>
-    <row r="45" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A45" s="8"/>
       <c r="B45" s="9"/>
       <c r="C45" s="10"/>
@@ -3026,7 +3086,7 @@
       <c r="AB45" s="13"/>
       <c r="AC45" s="13"/>
     </row>
-    <row r="46" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A46" s="8"/>
       <c r="B46" s="9"/>
       <c r="C46" s="10"/>
@@ -3056,7 +3116,7 @@
       <c r="AB46" s="13"/>
       <c r="AC46" s="13"/>
     </row>
-    <row r="47" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A47" s="8"/>
       <c r="B47" s="9"/>
       <c r="C47" s="10"/>
@@ -3086,7 +3146,7 @@
       <c r="AB47" s="13"/>
       <c r="AC47" s="13"/>
     </row>
-    <row r="48" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A48" s="8"/>
       <c r="B48" s="9"/>
       <c r="C48" s="10"/>
@@ -3116,7 +3176,7 @@
       <c r="AB48" s="13"/>
       <c r="AC48" s="13"/>
     </row>
-    <row r="49" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A49" s="8"/>
       <c r="B49" s="9"/>
       <c r="C49" s="10"/>
@@ -3146,7 +3206,7 @@
       <c r="AB49" s="13"/>
       <c r="AC49" s="13"/>
     </row>
-    <row r="50" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A50" s="8"/>
       <c r="B50" s="9"/>
       <c r="C50" s="10"/>
@@ -3176,7 +3236,7 @@
       <c r="AB50" s="13"/>
       <c r="AC50" s="13"/>
     </row>
-    <row r="51" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A51" s="8"/>
       <c r="B51" s="9"/>
       <c r="C51" s="10"/>
@@ -3206,7 +3266,7 @@
       <c r="AB51" s="13"/>
       <c r="AC51" s="13"/>
     </row>
-    <row r="52" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A52" s="8"/>
       <c r="B52" s="9"/>
       <c r="C52" s="10"/>
@@ -3236,7 +3296,7 @@
       <c r="AB52" s="13"/>
       <c r="AC52" s="13"/>
     </row>
-    <row r="53" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A53" s="8"/>
       <c r="B53" s="9"/>
       <c r="C53" s="10"/>
@@ -3266,7 +3326,7 @@
       <c r="AB53" s="13"/>
       <c r="AC53" s="13"/>
     </row>
-    <row r="54" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A54" s="8"/>
       <c r="B54" s="9"/>
       <c r="C54" s="10"/>
@@ -3296,7 +3356,7 @@
       <c r="AB54" s="13"/>
       <c r="AC54" s="13"/>
     </row>
-    <row r="55" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A55" s="8"/>
       <c r="B55" s="9"/>
       <c r="C55" s="10"/>
@@ -3326,7 +3386,7 @@
       <c r="AB55" s="13"/>
       <c r="AC55" s="13"/>
     </row>
-    <row r="56" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A56" s="8"/>
       <c r="B56" s="9"/>
       <c r="C56" s="10"/>
@@ -3356,7 +3416,7 @@
       <c r="AB56" s="13"/>
       <c r="AC56" s="13"/>
     </row>
-    <row r="57" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A57" s="8"/>
       <c r="B57" s="9"/>
       <c r="C57" s="10"/>
@@ -3386,7 +3446,7 @@
       <c r="AB57" s="13"/>
       <c r="AC57" s="13"/>
     </row>
-    <row r="58" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A58" s="8"/>
       <c r="B58" s="9"/>
       <c r="C58" s="10"/>
@@ -3416,7 +3476,7 @@
       <c r="AB58" s="13"/>
       <c r="AC58" s="13"/>
     </row>
-    <row r="59" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A59" s="8"/>
       <c r="B59" s="9"/>
       <c r="C59" s="10"/>
@@ -3446,7 +3506,7 @@
       <c r="AB59" s="13"/>
       <c r="AC59" s="13"/>
     </row>
-    <row r="60" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A60" s="8"/>
       <c r="B60" s="9"/>
       <c r="C60" s="10"/>
@@ -3476,7 +3536,7 @@
       <c r="AB60" s="13"/>
       <c r="AC60" s="13"/>
     </row>
-    <row r="61" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A61" s="8"/>
       <c r="B61" s="9"/>
       <c r="C61" s="10"/>
@@ -3506,7 +3566,7 @@
       <c r="AB61" s="13"/>
       <c r="AC61" s="13"/>
     </row>
-    <row r="62" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A62" s="8"/>
       <c r="B62" s="9"/>
       <c r="C62" s="10"/>
@@ -3536,7 +3596,7 @@
       <c r="AB62" s="13"/>
       <c r="AC62" s="13"/>
     </row>
-    <row r="63" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A63" s="8"/>
       <c r="B63" s="9"/>
       <c r="C63" s="10"/>
@@ -3566,7 +3626,7 @@
       <c r="AB63" s="13"/>
       <c r="AC63" s="13"/>
     </row>
-    <row r="64" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A64" s="8"/>
       <c r="B64" s="9"/>
       <c r="C64" s="10"/>
@@ -3596,7 +3656,7 @@
       <c r="AB64" s="13"/>
       <c r="AC64" s="13"/>
     </row>
-    <row r="65" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A65" s="8"/>
       <c r="B65" s="9"/>
       <c r="C65" s="10"/>
@@ -3626,7 +3686,7 @@
       <c r="AB65" s="13"/>
       <c r="AC65" s="13"/>
     </row>
-    <row r="66" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A66" s="8"/>
       <c r="B66" s="9"/>
       <c r="C66" s="10"/>
@@ -3656,7 +3716,7 @@
       <c r="AB66" s="13"/>
       <c r="AC66" s="13"/>
     </row>
-    <row r="67" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A67" s="8"/>
       <c r="B67" s="9"/>
       <c r="C67" s="10"/>
@@ -3686,7 +3746,7 @@
       <c r="AB67" s="13"/>
       <c r="AC67" s="13"/>
     </row>
-    <row r="68" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A68" s="8"/>
       <c r="B68" s="9"/>
       <c r="C68" s="10"/>
@@ -3716,7 +3776,7 @@
       <c r="AB68" s="13"/>
       <c r="AC68" s="13"/>
     </row>
-    <row r="69" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A69" s="8"/>
       <c r="B69" s="9"/>
       <c r="C69" s="10"/>
@@ -3746,7 +3806,7 @@
       <c r="AB69" s="13"/>
       <c r="AC69" s="13"/>
     </row>
-    <row r="70" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A70" s="8"/>
       <c r="B70" s="9"/>
       <c r="C70" s="10"/>
@@ -3776,7 +3836,7 @@
       <c r="AB70" s="13"/>
       <c r="AC70" s="13"/>
     </row>
-    <row r="71" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A71" s="8"/>
       <c r="B71" s="9"/>
       <c r="C71" s="10"/>
@@ -3806,7 +3866,7 @@
       <c r="AB71" s="13"/>
       <c r="AC71" s="13"/>
     </row>
-    <row r="72" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A72" s="8"/>
       <c r="B72" s="9"/>
       <c r="C72" s="10"/>
@@ -3836,7 +3896,7 @@
       <c r="AB72" s="13"/>
       <c r="AC72" s="13"/>
     </row>
-    <row r="73" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A73" s="8"/>
       <c r="B73" s="9"/>
       <c r="C73" s="10"/>
@@ -3866,7 +3926,7 @@
       <c r="AB73" s="13"/>
       <c r="AC73" s="13"/>
     </row>
-    <row r="74" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A74" s="8"/>
       <c r="B74" s="9"/>
       <c r="C74" s="10"/>
@@ -3896,7 +3956,7 @@
       <c r="AB74" s="13"/>
       <c r="AC74" s="13"/>
     </row>
-    <row r="75" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A75" s="8"/>
       <c r="B75" s="9"/>
       <c r="C75" s="10"/>
@@ -3926,7 +3986,7 @@
       <c r="AB75" s="13"/>
       <c r="AC75" s="13"/>
     </row>
-    <row r="76" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A76" s="8"/>
       <c r="B76" s="9"/>
       <c r="C76" s="10"/>
@@ -3956,7 +4016,7 @@
       <c r="AB76" s="13"/>
       <c r="AC76" s="13"/>
     </row>
-    <row r="77" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A77" s="8"/>
       <c r="B77" s="9"/>
       <c r="C77" s="10"/>
@@ -3986,7 +4046,7 @@
       <c r="AB77" s="13"/>
       <c r="AC77" s="13"/>
     </row>
-    <row r="78" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A78" s="8"/>
       <c r="B78" s="9"/>
       <c r="C78" s="10"/>
@@ -4016,7 +4076,7 @@
       <c r="AB78" s="13"/>
       <c r="AC78" s="13"/>
     </row>
-    <row r="79" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A79" s="8"/>
       <c r="B79" s="9"/>
       <c r="C79" s="10"/>
@@ -4046,7 +4106,7 @@
       <c r="AB79" s="13"/>
       <c r="AC79" s="13"/>
     </row>
-    <row r="80" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A80" s="8"/>
       <c r="B80" s="9"/>
       <c r="C80" s="10"/>
@@ -4076,7 +4136,7 @@
       <c r="AB80" s="13"/>
       <c r="AC80" s="13"/>
     </row>
-    <row r="81" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A81" s="8"/>
       <c r="B81" s="9"/>
       <c r="C81" s="10"/>
@@ -4106,7 +4166,7 @@
       <c r="AB81" s="13"/>
       <c r="AC81" s="13"/>
     </row>
-    <row r="82" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A82" s="8"/>
       <c r="B82" s="9"/>
       <c r="C82" s="10"/>
@@ -4136,7 +4196,7 @@
       <c r="AB82" s="13"/>
       <c r="AC82" s="13"/>
     </row>
-    <row r="83" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A83" s="8"/>
       <c r="B83" s="9"/>
       <c r="C83" s="10"/>
@@ -4166,7 +4226,7 @@
       <c r="AB83" s="13"/>
       <c r="AC83" s="13"/>
     </row>
-    <row r="84" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A84" s="8"/>
       <c r="B84" s="9"/>
       <c r="C84" s="10"/>
@@ -4196,7 +4256,7 @@
       <c r="AB84" s="13"/>
       <c r="AC84" s="13"/>
     </row>
-    <row r="85" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A85" s="8"/>
       <c r="B85" s="9"/>
       <c r="C85" s="10"/>
@@ -4226,7 +4286,7 @@
       <c r="AB85" s="13"/>
       <c r="AC85" s="13"/>
     </row>
-    <row r="86" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A86" s="8"/>
       <c r="B86" s="9"/>
       <c r="C86" s="10"/>
@@ -4256,7 +4316,7 @@
       <c r="AB86" s="13"/>
       <c r="AC86" s="13"/>
     </row>
-    <row r="87" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A87" s="8"/>
       <c r="B87" s="9"/>
       <c r="C87" s="10"/>
@@ -4286,7 +4346,7 @@
       <c r="AB87" s="13"/>
       <c r="AC87" s="13"/>
     </row>
-    <row r="88" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A88" s="8"/>
       <c r="B88" s="9"/>
       <c r="C88" s="10"/>
@@ -4316,7 +4376,7 @@
       <c r="AB88" s="13"/>
       <c r="AC88" s="13"/>
     </row>
-    <row r="89" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A89" s="8"/>
       <c r="B89" s="9"/>
       <c r="C89" s="10"/>
@@ -4346,7 +4406,7 @@
       <c r="AB89" s="13"/>
       <c r="AC89" s="13"/>
     </row>
-    <row r="90" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A90" s="8"/>
       <c r="B90" s="9"/>
       <c r="C90" s="10"/>
@@ -4376,7 +4436,7 @@
       <c r="AB90" s="13"/>
       <c r="AC90" s="13"/>
     </row>
-    <row r="91" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A91" s="8"/>
       <c r="B91" s="9"/>
       <c r="C91" s="10"/>
@@ -4406,7 +4466,7 @@
       <c r="AB91" s="13"/>
       <c r="AC91" s="13"/>
     </row>
-    <row r="92" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A92" s="8"/>
       <c r="B92" s="9"/>
       <c r="C92" s="10"/>
@@ -4436,7 +4496,7 @@
       <c r="AB92" s="13"/>
       <c r="AC92" s="13"/>
     </row>
-    <row r="93" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A93" s="8"/>
       <c r="B93" s="9"/>
       <c r="C93" s="10"/>
@@ -4466,7 +4526,7 @@
       <c r="AB93" s="13"/>
       <c r="AC93" s="13"/>
     </row>
-    <row r="94" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A94" s="8"/>
       <c r="B94" s="9"/>
       <c r="C94" s="10"/>
@@ -4496,7 +4556,7 @@
       <c r="AB94" s="13"/>
       <c r="AC94" s="13"/>
     </row>
-    <row r="95" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A95" s="8"/>
       <c r="B95" s="9"/>
       <c r="C95" s="10"/>
@@ -4526,7 +4586,7 @@
       <c r="AB95" s="13"/>
       <c r="AC95" s="13"/>
     </row>
-    <row r="96" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A96" s="8"/>
       <c r="B96" s="9"/>
       <c r="C96" s="10"/>
@@ -4556,7 +4616,7 @@
       <c r="AB96" s="13"/>
       <c r="AC96" s="13"/>
     </row>
-    <row r="97" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A97" s="8"/>
       <c r="B97" s="9"/>
       <c r="C97" s="10"/>
@@ -4586,7 +4646,7 @@
       <c r="AB97" s="13"/>
       <c r="AC97" s="13"/>
     </row>
-    <row r="98" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A98" s="8"/>
       <c r="B98" s="9"/>
       <c r="C98" s="10"/>
@@ -4616,7 +4676,7 @@
       <c r="AB98" s="13"/>
       <c r="AC98" s="13"/>
     </row>
-    <row r="99" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A99" s="8"/>
       <c r="B99" s="9"/>
       <c r="C99" s="10"/>
@@ -4646,7 +4706,7 @@
       <c r="AB99" s="13"/>
       <c r="AC99" s="13"/>
     </row>
-    <row r="100" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A100" s="8"/>
       <c r="B100" s="9"/>
       <c r="C100" s="10"/>
@@ -4676,7 +4736,7 @@
       <c r="AB100" s="13"/>
       <c r="AC100" s="13"/>
     </row>
-    <row r="101" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A101" s="8"/>
       <c r="B101" s="9"/>
       <c r="C101" s="10"/>
@@ -4706,7 +4766,7 @@
       <c r="AB101" s="13"/>
       <c r="AC101" s="13"/>
     </row>
-    <row r="102" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A102" s="8"/>
       <c r="B102" s="9"/>
       <c r="C102" s="10"/>
@@ -4736,7 +4796,7 @@
       <c r="AB102" s="13"/>
       <c r="AC102" s="13"/>
     </row>
-    <row r="103" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A103" s="8"/>
       <c r="B103" s="9"/>
       <c r="C103" s="10"/>
@@ -4766,7 +4826,7 @@
       <c r="AB103" s="13"/>
       <c r="AC103" s="13"/>
     </row>
-    <row r="104" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A104" s="8"/>
       <c r="B104" s="9"/>
       <c r="C104" s="10"/>
@@ -4796,7 +4856,7 @@
       <c r="AB104" s="13"/>
       <c r="AC104" s="13"/>
     </row>
-    <row r="105" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A105" s="8"/>
       <c r="B105" s="9"/>
       <c r="C105" s="10"/>
@@ -4826,7 +4886,7 @@
       <c r="AB105" s="13"/>
       <c r="AC105" s="13"/>
     </row>
-    <row r="106" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A106" s="8"/>
       <c r="B106" s="9"/>
       <c r="C106" s="10"/>
@@ -4856,7 +4916,7 @@
       <c r="AB106" s="13"/>
       <c r="AC106" s="13"/>
     </row>
-    <row r="107" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A107" s="8"/>
       <c r="B107" s="9"/>
       <c r="C107" s="10"/>
@@ -4886,7 +4946,7 @@
       <c r="AB107" s="13"/>
       <c r="AC107" s="13"/>
     </row>
-    <row r="108" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A108" s="8"/>
       <c r="B108" s="9"/>
       <c r="C108" s="10"/>
@@ -4916,7 +4976,7 @@
       <c r="AB108" s="13"/>
       <c r="AC108" s="13"/>
     </row>
-    <row r="109" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A109" s="8"/>
       <c r="B109" s="9"/>
       <c r="C109" s="10"/>
@@ -4946,7 +5006,7 @@
       <c r="AB109" s="13"/>
       <c r="AC109" s="13"/>
     </row>
-    <row r="110" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A110" s="8"/>
       <c r="B110" s="9"/>
       <c r="C110" s="10"/>
@@ -4976,7 +5036,7 @@
       <c r="AB110" s="13"/>
       <c r="AC110" s="13"/>
     </row>
-    <row r="111" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A111" s="8"/>
       <c r="B111" s="9"/>
       <c r="C111" s="10"/>
@@ -5006,7 +5066,7 @@
       <c r="AB111" s="13"/>
       <c r="AC111" s="13"/>
     </row>
-    <row r="112" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A112" s="8"/>
       <c r="B112" s="9"/>
       <c r="C112" s="10"/>
@@ -5036,7 +5096,7 @@
       <c r="AB112" s="13"/>
       <c r="AC112" s="13"/>
     </row>
-    <row r="113" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A113" s="8"/>
       <c r="B113" s="9"/>
       <c r="C113" s="10"/>
@@ -5066,7 +5126,7 @@
       <c r="AB113" s="13"/>
       <c r="AC113" s="13"/>
     </row>
-    <row r="114" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A114" s="8"/>
       <c r="B114" s="9"/>
       <c r="C114" s="10"/>
@@ -5096,7 +5156,7 @@
       <c r="AB114" s="13"/>
       <c r="AC114" s="13"/>
     </row>
-    <row r="115" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A115" s="8"/>
       <c r="B115" s="9"/>
       <c r="C115" s="10"/>
@@ -5126,7 +5186,7 @@
       <c r="AB115" s="13"/>
       <c r="AC115" s="13"/>
     </row>
-    <row r="116" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A116" s="8"/>
       <c r="B116" s="9"/>
       <c r="C116" s="10"/>
@@ -5156,7 +5216,7 @@
       <c r="AB116" s="13"/>
       <c r="AC116" s="13"/>
     </row>
-    <row r="117" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A117" s="8"/>
       <c r="B117" s="9"/>
       <c r="C117" s="10"/>
@@ -5186,7 +5246,7 @@
       <c r="AB117" s="13"/>
       <c r="AC117" s="13"/>
     </row>
-    <row r="118" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A118" s="8"/>
       <c r="B118" s="9"/>
       <c r="C118" s="10"/>
@@ -5216,7 +5276,7 @@
       <c r="AB118" s="13"/>
       <c r="AC118" s="13"/>
     </row>
-    <row r="119" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A119" s="8"/>
       <c r="B119" s="9"/>
       <c r="C119" s="10"/>
@@ -5246,7 +5306,7 @@
       <c r="AB119" s="13"/>
       <c r="AC119" s="13"/>
     </row>
-    <row r="120" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A120" s="8"/>
       <c r="B120" s="9"/>
       <c r="C120" s="10"/>
@@ -5276,7 +5336,7 @@
       <c r="AB120" s="13"/>
       <c r="AC120" s="13"/>
     </row>
-    <row r="121" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A121" s="8"/>
       <c r="B121" s="9"/>
       <c r="C121" s="10"/>
@@ -5306,7 +5366,7 @@
       <c r="AB121" s="13"/>
       <c r="AC121" s="13"/>
     </row>
-    <row r="122" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A122" s="8"/>
       <c r="B122" s="9"/>
       <c r="C122" s="10"/>
@@ -5336,7 +5396,7 @@
       <c r="AB122" s="13"/>
       <c r="AC122" s="13"/>
     </row>
-    <row r="123" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A123" s="8"/>
       <c r="B123" s="9"/>
       <c r="C123" s="10"/>
@@ -5366,7 +5426,7 @@
       <c r="AB123" s="13"/>
       <c r="AC123" s="13"/>
     </row>
-    <row r="124" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A124" s="8"/>
       <c r="B124" s="9"/>
       <c r="C124" s="10"/>
@@ -5396,7 +5456,7 @@
       <c r="AB124" s="13"/>
       <c r="AC124" s="13"/>
     </row>
-    <row r="125" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A125" s="8"/>
       <c r="B125" s="9"/>
       <c r="C125" s="10"/>
@@ -5426,7 +5486,7 @@
       <c r="AB125" s="13"/>
       <c r="AC125" s="13"/>
     </row>
-    <row r="126" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A126" s="8"/>
       <c r="B126" s="9"/>
       <c r="C126" s="10"/>
@@ -5456,7 +5516,7 @@
       <c r="AB126" s="13"/>
       <c r="AC126" s="13"/>
     </row>
-    <row r="127" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A127" s="8"/>
       <c r="B127" s="9"/>
       <c r="C127" s="10"/>
@@ -5486,7 +5546,7 @@
       <c r="AB127" s="13"/>
       <c r="AC127" s="13"/>
     </row>
-    <row r="128" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A128" s="8"/>
       <c r="B128" s="9"/>
       <c r="C128" s="10"/>
@@ -5516,7 +5576,7 @@
       <c r="AB128" s="13"/>
       <c r="AC128" s="13"/>
     </row>
-    <row r="129" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A129" s="8"/>
       <c r="B129" s="9"/>
       <c r="C129" s="10"/>
@@ -5546,7 +5606,7 @@
       <c r="AB129" s="13"/>
       <c r="AC129" s="13"/>
     </row>
-    <row r="130" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A130" s="8"/>
       <c r="B130" s="9"/>
       <c r="C130" s="10"/>
@@ -5576,7 +5636,7 @@
       <c r="AB130" s="13"/>
       <c r="AC130" s="13"/>
     </row>
-    <row r="131" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A131" s="8"/>
       <c r="B131" s="9"/>
       <c r="C131" s="10"/>
@@ -5606,7 +5666,7 @@
       <c r="AB131" s="13"/>
       <c r="AC131" s="13"/>
     </row>
-    <row r="132" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A132" s="8"/>
       <c r="B132" s="9"/>
       <c r="C132" s="10"/>
@@ -5636,7 +5696,7 @@
       <c r="AB132" s="13"/>
       <c r="AC132" s="13"/>
     </row>
-    <row r="133" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A133" s="8"/>
       <c r="B133" s="9"/>
       <c r="C133" s="10"/>
@@ -5666,7 +5726,7 @@
       <c r="AB133" s="13"/>
       <c r="AC133" s="13"/>
     </row>
-    <row r="134" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A134" s="8"/>
       <c r="B134" s="9"/>
       <c r="C134" s="10"/>
@@ -5696,7 +5756,7 @@
       <c r="AB134" s="13"/>
       <c r="AC134" s="13"/>
     </row>
-    <row r="135" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A135" s="8"/>
       <c r="B135" s="9"/>
       <c r="C135" s="10"/>
@@ -5726,7 +5786,7 @@
       <c r="AB135" s="13"/>
       <c r="AC135" s="13"/>
     </row>
-    <row r="136" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A136" s="8"/>
       <c r="B136" s="9"/>
       <c r="C136" s="10"/>
@@ -5756,7 +5816,7 @@
       <c r="AB136" s="13"/>
       <c r="AC136" s="13"/>
     </row>
-    <row r="137" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A137" s="8"/>
       <c r="B137" s="9"/>
       <c r="C137" s="10"/>
@@ -5786,7 +5846,7 @@
       <c r="AB137" s="13"/>
       <c r="AC137" s="13"/>
     </row>
-    <row r="138" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A138" s="8"/>
       <c r="B138" s="9"/>
       <c r="C138" s="10"/>
@@ -5816,7 +5876,7 @@
       <c r="AB138" s="13"/>
       <c r="AC138" s="13"/>
     </row>
-    <row r="139" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A139" s="8"/>
       <c r="B139" s="9"/>
       <c r="C139" s="10"/>
@@ -5846,7 +5906,7 @@
       <c r="AB139" s="13"/>
       <c r="AC139" s="13"/>
     </row>
-    <row r="140" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A140" s="8"/>
       <c r="B140" s="9"/>
       <c r="C140" s="10"/>
@@ -5876,7 +5936,7 @@
       <c r="AB140" s="13"/>
       <c r="AC140" s="13"/>
     </row>
-    <row r="141" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A141" s="8"/>
       <c r="B141" s="9"/>
       <c r="C141" s="10"/>
@@ -5906,7 +5966,7 @@
       <c r="AB141" s="13"/>
       <c r="AC141" s="13"/>
     </row>
-    <row r="142" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A142" s="8"/>
       <c r="B142" s="9"/>
       <c r="C142" s="10"/>
@@ -5936,7 +5996,7 @@
       <c r="AB142" s="13"/>
       <c r="AC142" s="13"/>
     </row>
-    <row r="143" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A143" s="8"/>
       <c r="B143" s="9"/>
       <c r="C143" s="10"/>
@@ -5966,7 +6026,7 @@
       <c r="AB143" s="13"/>
       <c r="AC143" s="13"/>
     </row>
-    <row r="144" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A144" s="8"/>
       <c r="B144" s="9"/>
       <c r="C144" s="10"/>
@@ -5996,7 +6056,7 @@
       <c r="AB144" s="13"/>
       <c r="AC144" s="13"/>
     </row>
-    <row r="145" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A145" s="8"/>
       <c r="B145" s="9"/>
       <c r="C145" s="10"/>
@@ -6026,7 +6086,7 @@
       <c r="AB145" s="13"/>
       <c r="AC145" s="13"/>
     </row>
-    <row r="146" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A146" s="8"/>
       <c r="B146" s="9"/>
       <c r="C146" s="10"/>
@@ -6056,7 +6116,7 @@
       <c r="AB146" s="13"/>
       <c r="AC146" s="13"/>
     </row>
-    <row r="147" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A147" s="8"/>
       <c r="B147" s="9"/>
       <c r="C147" s="10"/>
@@ -6086,7 +6146,7 @@
       <c r="AB147" s="13"/>
       <c r="AC147" s="13"/>
     </row>
-    <row r="148" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A148" s="8"/>
       <c r="B148" s="9"/>
       <c r="C148" s="10"/>
@@ -6116,7 +6176,7 @@
       <c r="AB148" s="13"/>
       <c r="AC148" s="13"/>
     </row>
-    <row r="149" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A149" s="8"/>
       <c r="B149" s="9"/>
       <c r="C149" s="10"/>
@@ -6146,7 +6206,7 @@
       <c r="AB149" s="13"/>
       <c r="AC149" s="13"/>
     </row>
-    <row r="150" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A150" s="8"/>
       <c r="B150" s="9"/>
       <c r="C150" s="10"/>
@@ -6176,7 +6236,7 @@
       <c r="AB150" s="13"/>
       <c r="AC150" s="13"/>
     </row>
-    <row r="151" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A151" s="8"/>
       <c r="B151" s="9"/>
       <c r="C151" s="10"/>
@@ -6206,7 +6266,7 @@
       <c r="AB151" s="13"/>
       <c r="AC151" s="13"/>
     </row>
-    <row r="152" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A152" s="8"/>
       <c r="B152" s="9"/>
       <c r="C152" s="10"/>
@@ -6236,7 +6296,7 @@
       <c r="AB152" s="13"/>
       <c r="AC152" s="13"/>
     </row>
-    <row r="153" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A153" s="8"/>
       <c r="B153" s="9"/>
       <c r="C153" s="10"/>
@@ -6266,7 +6326,7 @@
       <c r="AB153" s="13"/>
       <c r="AC153" s="13"/>
     </row>
-    <row r="154" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A154" s="8"/>
       <c r="B154" s="9"/>
       <c r="C154" s="10"/>
@@ -6296,7 +6356,7 @@
       <c r="AB154" s="13"/>
       <c r="AC154" s="13"/>
     </row>
-    <row r="155" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A155" s="8"/>
       <c r="B155" s="9"/>
       <c r="C155" s="10"/>
@@ -6326,7 +6386,7 @@
       <c r="AB155" s="13"/>
       <c r="AC155" s="13"/>
     </row>
-    <row r="156" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A156" s="8"/>
       <c r="B156" s="9"/>
       <c r="C156" s="10"/>
@@ -6356,7 +6416,7 @@
       <c r="AB156" s="13"/>
       <c r="AC156" s="13"/>
     </row>
-    <row r="157" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A157" s="8"/>
       <c r="B157" s="9"/>
       <c r="C157" s="10"/>
@@ -6386,7 +6446,7 @@
       <c r="AB157" s="13"/>
       <c r="AC157" s="13"/>
     </row>
-    <row r="158" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A158" s="8"/>
       <c r="B158" s="9"/>
       <c r="C158" s="10"/>
@@ -6416,7 +6476,7 @@
       <c r="AB158" s="13"/>
       <c r="AC158" s="13"/>
     </row>
-    <row r="159" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A159" s="8"/>
       <c r="B159" s="9"/>
       <c r="C159" s="10"/>
@@ -6446,7 +6506,7 @@
       <c r="AB159" s="13"/>
       <c r="AC159" s="13"/>
     </row>
-    <row r="160" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A160" s="8"/>
       <c r="B160" s="9"/>
       <c r="C160" s="10"/>
@@ -6476,7 +6536,7 @@
       <c r="AB160" s="13"/>
       <c r="AC160" s="13"/>
     </row>
-    <row r="161" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A161" s="8"/>
       <c r="B161" s="9"/>
       <c r="C161" s="10"/>
@@ -6506,7 +6566,7 @@
       <c r="AB161" s="13"/>
       <c r="AC161" s="13"/>
     </row>
-    <row r="162" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A162" s="8"/>
       <c r="B162" s="9"/>
       <c r="C162" s="10"/>
@@ -6536,7 +6596,7 @@
       <c r="AB162" s="13"/>
       <c r="AC162" s="13"/>
     </row>
-    <row r="163" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A163" s="8"/>
       <c r="B163" s="9"/>
       <c r="C163" s="10"/>
@@ -6566,7 +6626,7 @@
       <c r="AB163" s="13"/>
       <c r="AC163" s="13"/>
     </row>
-    <row r="164" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A164" s="8"/>
       <c r="B164" s="9"/>
       <c r="C164" s="10"/>
@@ -6596,7 +6656,7 @@
       <c r="AB164" s="13"/>
       <c r="AC164" s="13"/>
     </row>
-    <row r="165" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A165" s="8"/>
       <c r="B165" s="9"/>
       <c r="C165" s="10"/>
@@ -6626,7 +6686,7 @@
       <c r="AB165" s="13"/>
       <c r="AC165" s="13"/>
     </row>
-    <row r="166" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A166" s="8"/>
       <c r="B166" s="9"/>
       <c r="C166" s="10"/>
@@ -6656,7 +6716,7 @@
       <c r="AB166" s="13"/>
       <c r="AC166" s="13"/>
     </row>
-    <row r="167" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A167" s="8"/>
       <c r="B167" s="9"/>
       <c r="C167" s="10"/>
@@ -6686,7 +6746,7 @@
       <c r="AB167" s="13"/>
       <c r="AC167" s="13"/>
     </row>
-    <row r="168" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A168" s="8"/>
       <c r="B168" s="9"/>
       <c r="C168" s="10"/>
@@ -6716,7 +6776,7 @@
       <c r="AB168" s="13"/>
       <c r="AC168" s="13"/>
     </row>
-    <row r="169" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A169" s="8"/>
       <c r="B169" s="9"/>
       <c r="C169" s="10"/>
@@ -6746,7 +6806,7 @@
       <c r="AB169" s="13"/>
       <c r="AC169" s="13"/>
     </row>
-    <row r="170" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A170" s="8"/>
       <c r="B170" s="9"/>
       <c r="C170" s="10"/>
@@ -6776,7 +6836,7 @@
       <c r="AB170" s="13"/>
       <c r="AC170" s="13"/>
     </row>
-    <row r="171" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A171" s="8"/>
       <c r="B171" s="9"/>
       <c r="C171" s="10"/>
@@ -6806,7 +6866,7 @@
       <c r="AB171" s="13"/>
       <c r="AC171" s="13"/>
     </row>
-    <row r="172" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A172" s="8"/>
       <c r="B172" s="9"/>
       <c r="C172" s="10"/>
@@ -6836,7 +6896,7 @@
       <c r="AB172" s="13"/>
       <c r="AC172" s="13"/>
     </row>
-    <row r="173" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A173" s="8"/>
       <c r="B173" s="9"/>
       <c r="C173" s="10"/>
@@ -6866,7 +6926,7 @@
       <c r="AB173" s="13"/>
       <c r="AC173" s="13"/>
     </row>
-    <row r="174" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A174" s="8"/>
       <c r="B174" s="9"/>
       <c r="C174" s="10"/>
@@ -6896,7 +6956,7 @@
       <c r="AB174" s="13"/>
       <c r="AC174" s="13"/>
     </row>
-    <row r="175" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A175" s="8"/>
       <c r="B175" s="9"/>
       <c r="C175" s="10"/>
@@ -6926,7 +6986,7 @@
       <c r="AB175" s="13"/>
       <c r="AC175" s="13"/>
     </row>
-    <row r="176" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A176" s="8"/>
       <c r="B176" s="9"/>
       <c r="C176" s="10"/>
@@ -6956,7 +7016,7 @@
       <c r="AB176" s="13"/>
       <c r="AC176" s="13"/>
     </row>
-    <row r="177" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A177" s="8"/>
       <c r="B177" s="9"/>
       <c r="C177" s="10"/>
@@ -6986,7 +7046,7 @@
       <c r="AB177" s="13"/>
       <c r="AC177" s="13"/>
     </row>
-    <row r="178" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A178" s="8"/>
       <c r="B178" s="9"/>
       <c r="C178" s="10"/>
@@ -7016,7 +7076,7 @@
       <c r="AB178" s="13"/>
       <c r="AC178" s="13"/>
     </row>
-    <row r="179" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A179" s="8"/>
       <c r="B179" s="9"/>
       <c r="C179" s="10"/>
@@ -7046,7 +7106,7 @@
       <c r="AB179" s="13"/>
       <c r="AC179" s="13"/>
     </row>
-    <row r="180" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A180" s="8"/>
       <c r="B180" s="9"/>
       <c r="C180" s="10"/>
@@ -7076,7 +7136,7 @@
       <c r="AB180" s="13"/>
       <c r="AC180" s="13"/>
     </row>
-    <row r="181" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A181" s="8"/>
       <c r="B181" s="9"/>
       <c r="C181" s="10"/>
@@ -7106,7 +7166,7 @@
       <c r="AB181" s="13"/>
       <c r="AC181" s="13"/>
     </row>
-    <row r="182" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A182" s="8"/>
       <c r="B182" s="9"/>
       <c r="C182" s="10"/>
@@ -7136,7 +7196,7 @@
       <c r="AB182" s="13"/>
       <c r="AC182" s="13"/>
     </row>
-    <row r="183" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A183" s="8"/>
       <c r="B183" s="9"/>
       <c r="C183" s="10"/>
@@ -7166,7 +7226,7 @@
       <c r="AB183" s="13"/>
       <c r="AC183" s="13"/>
     </row>
-    <row r="184" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A184" s="8"/>
       <c r="B184" s="9"/>
       <c r="C184" s="10"/>
@@ -7196,7 +7256,7 @@
       <c r="AB184" s="13"/>
       <c r="AC184" s="13"/>
     </row>
-    <row r="185" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A185" s="8"/>
       <c r="B185" s="9"/>
       <c r="C185" s="10"/>
@@ -7226,7 +7286,7 @@
       <c r="AB185" s="13"/>
       <c r="AC185" s="13"/>
     </row>
-    <row r="186" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A186" s="8"/>
       <c r="B186" s="9"/>
       <c r="C186" s="10"/>
@@ -7256,7 +7316,7 @@
       <c r="AB186" s="13"/>
       <c r="AC186" s="13"/>
     </row>
-    <row r="187" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A187" s="8"/>
       <c r="B187" s="9"/>
       <c r="C187" s="10"/>
@@ -7286,7 +7346,7 @@
       <c r="AB187" s="13"/>
       <c r="AC187" s="13"/>
     </row>
-    <row r="188" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A188" s="8"/>
       <c r="B188" s="9"/>
       <c r="C188" s="10"/>
@@ -7316,7 +7376,7 @@
       <c r="AB188" s="13"/>
       <c r="AC188" s="13"/>
     </row>
-    <row r="189" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A189" s="8"/>
       <c r="B189" s="9"/>
       <c r="C189" s="10"/>
@@ -7346,7 +7406,7 @@
       <c r="AB189" s="13"/>
       <c r="AC189" s="13"/>
     </row>
-    <row r="190" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A190" s="8"/>
       <c r="B190" s="9"/>
       <c r="C190" s="10"/>
@@ -7376,7 +7436,7 @@
       <c r="AB190" s="13"/>
       <c r="AC190" s="13"/>
     </row>
-    <row r="191" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A191" s="8"/>
       <c r="B191" s="9"/>
       <c r="C191" s="10"/>
@@ -7406,7 +7466,7 @@
       <c r="AB191" s="13"/>
       <c r="AC191" s="13"/>
     </row>
-    <row r="192" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A192" s="8"/>
       <c r="B192" s="9"/>
       <c r="C192" s="10"/>
@@ -7436,7 +7496,7 @@
       <c r="AB192" s="13"/>
       <c r="AC192" s="13"/>
     </row>
-    <row r="193" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A193" s="8"/>
       <c r="B193" s="9"/>
       <c r="C193" s="10"/>
@@ -7466,7 +7526,7 @@
       <c r="AB193" s="13"/>
       <c r="AC193" s="13"/>
     </row>
-    <row r="194" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A194" s="8"/>
       <c r="B194" s="9"/>
       <c r="C194" s="10"/>
@@ -7496,7 +7556,7 @@
       <c r="AB194" s="13"/>
       <c r="AC194" s="13"/>
     </row>
-    <row r="195" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A195" s="8"/>
       <c r="B195" s="9"/>
       <c r="C195" s="10"/>
@@ -7526,7 +7586,7 @@
       <c r="AB195" s="13"/>
       <c r="AC195" s="13"/>
     </row>
-    <row r="196" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A196" s="8"/>
       <c r="B196" s="9"/>
       <c r="C196" s="10"/>
@@ -7556,7 +7616,7 @@
       <c r="AB196" s="13"/>
       <c r="AC196" s="13"/>
     </row>
-    <row r="197" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A197" s="8"/>
       <c r="B197" s="9"/>
       <c r="C197" s="10"/>
@@ -7586,7 +7646,7 @@
       <c r="AB197" s="13"/>
       <c r="AC197" s="13"/>
     </row>
-    <row r="198" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A198" s="8"/>
       <c r="B198" s="9"/>
       <c r="C198" s="10"/>
@@ -7616,7 +7676,7 @@
       <c r="AB198" s="13"/>
       <c r="AC198" s="13"/>
     </row>
-    <row r="199" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A199" s="8"/>
       <c r="B199" s="9"/>
       <c r="C199" s="10"/>
@@ -7646,7 +7706,7 @@
       <c r="AB199" s="13"/>
       <c r="AC199" s="13"/>
     </row>
-    <row r="200" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A200" s="8"/>
       <c r="B200" s="9"/>
       <c r="C200" s="10"/>
@@ -7676,7 +7736,7 @@
       <c r="AB200" s="13"/>
       <c r="AC200" s="13"/>
     </row>
-    <row r="201" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A201" s="8"/>
       <c r="B201" s="9"/>
       <c r="C201" s="10"/>
@@ -7706,7 +7766,7 @@
       <c r="AB201" s="13"/>
       <c r="AC201" s="13"/>
     </row>
-    <row r="202" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A202" s="8"/>
       <c r="B202" s="9"/>
       <c r="C202" s="10"/>
@@ -7736,7 +7796,7 @@
       <c r="AB202" s="13"/>
       <c r="AC202" s="13"/>
     </row>
-    <row r="203" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A203" s="8"/>
       <c r="B203" s="9"/>
       <c r="C203" s="10"/>
@@ -7766,7 +7826,7 @@
       <c r="AB203" s="13"/>
       <c r="AC203" s="13"/>
     </row>
-    <row r="204" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A204" s="8"/>
       <c r="B204" s="9"/>
       <c r="C204" s="10"/>
@@ -7796,7 +7856,7 @@
       <c r="AB204" s="13"/>
       <c r="AC204" s="13"/>
     </row>
-    <row r="205" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A205" s="8"/>
       <c r="B205" s="9"/>
       <c r="C205" s="10"/>
@@ -7826,7 +7886,7 @@
       <c r="AB205" s="13"/>
       <c r="AC205" s="13"/>
     </row>
-    <row r="206" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A206" s="8"/>
       <c r="B206" s="9"/>
       <c r="C206" s="10"/>
@@ -7856,7 +7916,7 @@
       <c r="AB206" s="13"/>
       <c r="AC206" s="13"/>
     </row>
-    <row r="207" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A207" s="8"/>
       <c r="B207" s="9"/>
       <c r="C207" s="10"/>
@@ -7886,7 +7946,7 @@
       <c r="AB207" s="13"/>
       <c r="AC207" s="13"/>
     </row>
-    <row r="208" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A208" s="8"/>
       <c r="B208" s="9"/>
       <c r="C208" s="10"/>
@@ -7916,7 +7976,7 @@
       <c r="AB208" s="13"/>
       <c r="AC208" s="13"/>
     </row>
-    <row r="209" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A209" s="8"/>
       <c r="B209" s="9"/>
       <c r="C209" s="10"/>
@@ -7946,7 +8006,7 @@
       <c r="AB209" s="13"/>
       <c r="AC209" s="13"/>
     </row>
-    <row r="210" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A210" s="8"/>
       <c r="B210" s="9"/>
       <c r="C210" s="10"/>
@@ -7976,7 +8036,7 @@
       <c r="AB210" s="13"/>
       <c r="AC210" s="13"/>
     </row>
-    <row r="211" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A211" s="8"/>
       <c r="B211" s="9"/>
       <c r="C211" s="10"/>
@@ -8006,7 +8066,7 @@
       <c r="AB211" s="13"/>
       <c r="AC211" s="13"/>
     </row>
-    <row r="212" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A212" s="8"/>
       <c r="B212" s="9"/>
       <c r="C212" s="10"/>
@@ -8036,7 +8096,7 @@
       <c r="AB212" s="13"/>
       <c r="AC212" s="13"/>
     </row>
-    <row r="213" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A213" s="8"/>
       <c r="B213" s="9"/>
       <c r="C213" s="10"/>
@@ -8066,7 +8126,7 @@
       <c r="AB213" s="13"/>
       <c r="AC213" s="13"/>
     </row>
-    <row r="214" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A214" s="8"/>
       <c r="B214" s="9"/>
       <c r="C214" s="10"/>
@@ -8096,7 +8156,7 @@
       <c r="AB214" s="13"/>
       <c r="AC214" s="13"/>
     </row>
-    <row r="215" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A215" s="8"/>
       <c r="B215" s="9"/>
       <c r="C215" s="10"/>
@@ -8126,7 +8186,7 @@
       <c r="AB215" s="13"/>
       <c r="AC215" s="13"/>
     </row>
-    <row r="216" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A216" s="8"/>
       <c r="B216" s="9"/>
       <c r="C216" s="10"/>
@@ -8156,7 +8216,7 @@
       <c r="AB216" s="13"/>
       <c r="AC216" s="13"/>
     </row>
-    <row r="217" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A217" s="8"/>
       <c r="B217" s="9"/>
       <c r="C217" s="10"/>
@@ -8186,7 +8246,7 @@
       <c r="AB217" s="13"/>
       <c r="AC217" s="13"/>
     </row>
-    <row r="218" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A218" s="8"/>
       <c r="B218" s="9"/>
       <c r="C218" s="10"/>
@@ -8216,7 +8276,7 @@
       <c r="AB218" s="13"/>
       <c r="AC218" s="13"/>
     </row>
-    <row r="219" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A219" s="8"/>
       <c r="B219" s="9"/>
       <c r="C219" s="10"/>
@@ -8246,7 +8306,7 @@
       <c r="AB219" s="13"/>
       <c r="AC219" s="13"/>
     </row>
-    <row r="220" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A220" s="8"/>
       <c r="B220" s="9"/>
       <c r="C220" s="10"/>
@@ -8276,7 +8336,7 @@
       <c r="AB220" s="13"/>
       <c r="AC220" s="13"/>
     </row>
-    <row r="221" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A221" s="8"/>
       <c r="B221" s="9"/>
       <c r="C221" s="10"/>
@@ -8306,7 +8366,7 @@
       <c r="AB221" s="13"/>
       <c r="AC221" s="13"/>
     </row>
-    <row r="222" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A222" s="8"/>
       <c r="B222" s="9"/>
       <c r="C222" s="10"/>
@@ -8336,7 +8396,7 @@
       <c r="AB222" s="13"/>
       <c r="AC222" s="13"/>
     </row>
-    <row r="223" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A223" s="8"/>
       <c r="B223" s="9"/>
       <c r="C223" s="10"/>
@@ -8366,7 +8426,7 @@
       <c r="AB223" s="13"/>
       <c r="AC223" s="13"/>
     </row>
-    <row r="224" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A224" s="8"/>
       <c r="B224" s="9"/>
       <c r="C224" s="10"/>
@@ -8396,7 +8456,7 @@
       <c r="AB224" s="13"/>
       <c r="AC224" s="13"/>
     </row>
-    <row r="225" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A225" s="8"/>
       <c r="B225" s="9"/>
       <c r="C225" s="10"/>
@@ -8426,7 +8486,7 @@
       <c r="AB225" s="13"/>
       <c r="AC225" s="13"/>
     </row>
-    <row r="226" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A226" s="8"/>
       <c r="B226" s="9"/>
       <c r="C226" s="10"/>
@@ -8456,7 +8516,7 @@
       <c r="AB226" s="13"/>
       <c r="AC226" s="13"/>
     </row>
-    <row r="227" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A227" s="8"/>
       <c r="B227" s="9"/>
       <c r="C227" s="10"/>
@@ -8486,7 +8546,7 @@
       <c r="AB227" s="13"/>
       <c r="AC227" s="13"/>
     </row>
-    <row r="228" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A228" s="8"/>
       <c r="B228" s="9"/>
       <c r="C228" s="10"/>
@@ -8516,7 +8576,7 @@
       <c r="AB228" s="13"/>
       <c r="AC228" s="13"/>
     </row>
-    <row r="229" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A229" s="8"/>
       <c r="B229" s="9"/>
       <c r="C229" s="10"/>
@@ -8546,7 +8606,7 @@
       <c r="AB229" s="13"/>
       <c r="AC229" s="13"/>
     </row>
-    <row r="230" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A230" s="8"/>
       <c r="B230" s="9"/>
       <c r="C230" s="10"/>
@@ -8576,7 +8636,7 @@
       <c r="AB230" s="13"/>
       <c r="AC230" s="13"/>
     </row>
-    <row r="231" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A231" s="8"/>
       <c r="B231" s="9"/>
       <c r="C231" s="10"/>
@@ -8606,7 +8666,7 @@
       <c r="AB231" s="13"/>
       <c r="AC231" s="13"/>
     </row>
-    <row r="232" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A232" s="8"/>
       <c r="B232" s="9"/>
       <c r="C232" s="10"/>
@@ -8636,7 +8696,7 @@
       <c r="AB232" s="13"/>
       <c r="AC232" s="13"/>
     </row>
-    <row r="233" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A233" s="8"/>
       <c r="B233" s="9"/>
       <c r="C233" s="10"/>
@@ -8666,7 +8726,7 @@
       <c r="AB233" s="13"/>
       <c r="AC233" s="13"/>
     </row>
-    <row r="234" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A234" s="8"/>
       <c r="B234" s="9"/>
       <c r="C234" s="10"/>
@@ -8696,7 +8756,7 @@
       <c r="AB234" s="13"/>
       <c r="AC234" s="13"/>
     </row>
-    <row r="235" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A235" s="8"/>
       <c r="B235" s="9"/>
       <c r="C235" s="10"/>
@@ -8726,7 +8786,7 @@
       <c r="AB235" s="13"/>
       <c r="AC235" s="13"/>
     </row>
-    <row r="236" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A236" s="8"/>
       <c r="B236" s="9"/>
       <c r="C236" s="10"/>
@@ -8756,7 +8816,7 @@
       <c r="AB236" s="13"/>
       <c r="AC236" s="13"/>
     </row>
-    <row r="237" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A237" s="8"/>
       <c r="B237" s="9"/>
       <c r="C237" s="10"/>
@@ -8786,7 +8846,7 @@
       <c r="AB237" s="13"/>
       <c r="AC237" s="13"/>
     </row>
-    <row r="238" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A238" s="8"/>
       <c r="B238" s="9"/>
       <c r="C238" s="10"/>
@@ -8816,7 +8876,7 @@
       <c r="AB238" s="13"/>
       <c r="AC238" s="13"/>
     </row>
-    <row r="239" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A239" s="8"/>
       <c r="B239" s="9"/>
       <c r="C239" s="10"/>
@@ -8846,7 +8906,7 @@
       <c r="AB239" s="13"/>
       <c r="AC239" s="13"/>
     </row>
-    <row r="240" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A240" s="8"/>
       <c r="B240" s="9"/>
       <c r="C240" s="10"/>
@@ -8876,7 +8936,7 @@
       <c r="AB240" s="13"/>
       <c r="AC240" s="13"/>
     </row>
-    <row r="241" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A241" s="8"/>
       <c r="B241" s="9"/>
       <c r="C241" s="10"/>
@@ -8906,7 +8966,7 @@
       <c r="AB241" s="13"/>
       <c r="AC241" s="13"/>
     </row>
-    <row r="242" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A242" s="8"/>
       <c r="B242" s="9"/>
       <c r="C242" s="10"/>
@@ -8936,7 +8996,7 @@
       <c r="AB242" s="13"/>
       <c r="AC242" s="13"/>
     </row>
-    <row r="243" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A243" s="8"/>
       <c r="B243" s="9"/>
       <c r="C243" s="10"/>
@@ -8966,7 +9026,7 @@
       <c r="AB243" s="13"/>
       <c r="AC243" s="13"/>
     </row>
-    <row r="244" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A244" s="8"/>
       <c r="B244" s="9"/>
       <c r="C244" s="10"/>
@@ -8996,7 +9056,7 @@
       <c r="AB244" s="13"/>
       <c r="AC244" s="13"/>
     </row>
-    <row r="245" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A245" s="8"/>
       <c r="B245" s="9"/>
       <c r="C245" s="10"/>
@@ -9026,7 +9086,7 @@
       <c r="AB245" s="13"/>
       <c r="AC245" s="13"/>
     </row>
-    <row r="246" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A246" s="8"/>
       <c r="B246" s="9"/>
       <c r="C246" s="10"/>
@@ -9056,7 +9116,7 @@
       <c r="AB246" s="13"/>
       <c r="AC246" s="13"/>
     </row>
-    <row r="247" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A247" s="8"/>
       <c r="B247" s="9"/>
       <c r="C247" s="10"/>
@@ -9086,7 +9146,7 @@
       <c r="AB247" s="13"/>
       <c r="AC247" s="13"/>
     </row>
-    <row r="248" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A248" s="8"/>
       <c r="B248" s="9"/>
       <c r="C248" s="10"/>
@@ -9116,7 +9176,7 @@
       <c r="AB248" s="13"/>
       <c r="AC248" s="13"/>
     </row>
-    <row r="249" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A249" s="8"/>
       <c r="B249" s="9"/>
       <c r="C249" s="10"/>
@@ -9146,7 +9206,7 @@
       <c r="AB249" s="13"/>
       <c r="AC249" s="13"/>
     </row>
-    <row r="250" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A250" s="8"/>
       <c r="B250" s="9"/>
       <c r="C250" s="10"/>
@@ -9176,7 +9236,7 @@
       <c r="AB250" s="13"/>
       <c r="AC250" s="13"/>
     </row>
-    <row r="251" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A251" s="8"/>
       <c r="B251" s="9"/>
       <c r="C251" s="10"/>
@@ -9206,7 +9266,7 @@
       <c r="AB251" s="13"/>
       <c r="AC251" s="13"/>
     </row>
-    <row r="252" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A252" s="8"/>
       <c r="B252" s="9"/>
       <c r="C252" s="10"/>
@@ -9236,7 +9296,7 @@
       <c r="AB252" s="13"/>
       <c r="AC252" s="13"/>
     </row>
-    <row r="253" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A253" s="8"/>
       <c r="B253" s="9"/>
       <c r="C253" s="10"/>
@@ -9266,7 +9326,7 @@
       <c r="AB253" s="13"/>
       <c r="AC253" s="13"/>
     </row>
-    <row r="254" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A254" s="8"/>
       <c r="B254" s="9"/>
       <c r="C254" s="10"/>
@@ -9296,7 +9356,7 @@
       <c r="AB254" s="13"/>
       <c r="AC254" s="13"/>
     </row>
-    <row r="255" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A255" s="8"/>
       <c r="B255" s="9"/>
       <c r="C255" s="10"/>
@@ -9326,7 +9386,7 @@
       <c r="AB255" s="13"/>
       <c r="AC255" s="13"/>
     </row>
-    <row r="256" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A256" s="8"/>
       <c r="B256" s="9"/>
       <c r="C256" s="10"/>
@@ -9356,7 +9416,7 @@
       <c r="AB256" s="13"/>
       <c r="AC256" s="13"/>
     </row>
-    <row r="257" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A257" s="8"/>
       <c r="B257" s="9"/>
       <c r="C257" s="10"/>
@@ -9386,7 +9446,7 @@
       <c r="AB257" s="13"/>
       <c r="AC257" s="13"/>
     </row>
-    <row r="258" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A258" s="8"/>
       <c r="B258" s="9"/>
       <c r="C258" s="10"/>
@@ -9416,7 +9476,7 @@
       <c r="AB258" s="13"/>
       <c r="AC258" s="13"/>
     </row>
-    <row r="259" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A259" s="8"/>
       <c r="B259" s="9"/>
       <c r="C259" s="10"/>
@@ -9446,7 +9506,7 @@
       <c r="AB259" s="13"/>
       <c r="AC259" s="13"/>
     </row>
-    <row r="260" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A260" s="8"/>
       <c r="B260" s="9"/>
       <c r="C260" s="10"/>
@@ -9476,7 +9536,7 @@
       <c r="AB260" s="13"/>
       <c r="AC260" s="13"/>
     </row>
-    <row r="261" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A261" s="8"/>
       <c r="B261" s="9"/>
       <c r="C261" s="10"/>
@@ -9506,7 +9566,7 @@
       <c r="AB261" s="13"/>
       <c r="AC261" s="13"/>
     </row>
-    <row r="262" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A262" s="8"/>
       <c r="B262" s="9"/>
       <c r="C262" s="10"/>
@@ -9536,7 +9596,7 @@
       <c r="AB262" s="13"/>
       <c r="AC262" s="13"/>
     </row>
-    <row r="263" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A263" s="8"/>
       <c r="B263" s="9"/>
       <c r="C263" s="10"/>
@@ -9566,7 +9626,7 @@
       <c r="AB263" s="13"/>
       <c r="AC263" s="13"/>
     </row>
-    <row r="264" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A264" s="8"/>
       <c r="B264" s="9"/>
       <c r="C264" s="10"/>
@@ -9596,7 +9656,7 @@
       <c r="AB264" s="13"/>
       <c r="AC264" s="13"/>
     </row>
-    <row r="265" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A265" s="8"/>
       <c r="B265" s="9"/>
       <c r="C265" s="10"/>
@@ -9626,7 +9686,7 @@
       <c r="AB265" s="13"/>
       <c r="AC265" s="13"/>
     </row>
-    <row r="266" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A266" s="8"/>
       <c r="B266" s="9"/>
       <c r="C266" s="10"/>
@@ -9656,7 +9716,7 @@
       <c r="AB266" s="13"/>
       <c r="AC266" s="13"/>
     </row>
-    <row r="267" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A267" s="8"/>
       <c r="B267" s="9"/>
       <c r="C267" s="10"/>
@@ -9686,7 +9746,7 @@
       <c r="AB267" s="13"/>
       <c r="AC267" s="13"/>
     </row>
-    <row r="268" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A268" s="8"/>
       <c r="B268" s="9"/>
       <c r="C268" s="10"/>
@@ -9716,7 +9776,7 @@
       <c r="AB268" s="13"/>
       <c r="AC268" s="13"/>
     </row>
-    <row r="269" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A269" s="8"/>
       <c r="B269" s="9"/>
       <c r="C269" s="10"/>
@@ -9746,7 +9806,7 @@
       <c r="AB269" s="13"/>
       <c r="AC269" s="13"/>
     </row>
-    <row r="270" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A270" s="8"/>
       <c r="B270" s="9"/>
       <c r="C270" s="10"/>
@@ -9776,7 +9836,7 @@
       <c r="AB270" s="13"/>
       <c r="AC270" s="13"/>
     </row>
-    <row r="271" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A271" s="8"/>
       <c r="B271" s="9"/>
       <c r="C271" s="10"/>
@@ -9806,7 +9866,7 @@
       <c r="AB271" s="13"/>
       <c r="AC271" s="13"/>
     </row>
-    <row r="272" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A272" s="8"/>
       <c r="B272" s="9"/>
       <c r="C272" s="10"/>
@@ -9836,7 +9896,7 @@
       <c r="AB272" s="13"/>
       <c r="AC272" s="13"/>
     </row>
-    <row r="273" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A273" s="8"/>
       <c r="B273" s="9"/>
       <c r="C273" s="10"/>
@@ -9866,7 +9926,7 @@
       <c r="AB273" s="13"/>
       <c r="AC273" s="13"/>
     </row>
-    <row r="274" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A274" s="8"/>
       <c r="B274" s="9"/>
       <c r="C274" s="10"/>
@@ -9896,7 +9956,7 @@
       <c r="AB274" s="13"/>
       <c r="AC274" s="13"/>
     </row>
-    <row r="275" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A275" s="8"/>
       <c r="B275" s="9"/>
       <c r="C275" s="10"/>
@@ -9926,7 +9986,7 @@
       <c r="AB275" s="13"/>
       <c r="AC275" s="13"/>
     </row>
-    <row r="276" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A276" s="8"/>
       <c r="B276" s="9"/>
       <c r="C276" s="10"/>
@@ -9956,7 +10016,7 @@
       <c r="AB276" s="13"/>
       <c r="AC276" s="13"/>
     </row>
-    <row r="277" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A277" s="8"/>
       <c r="B277" s="9"/>
       <c r="C277" s="10"/>
@@ -9986,7 +10046,7 @@
       <c r="AB277" s="13"/>
       <c r="AC277" s="13"/>
     </row>
-    <row r="278" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A278" s="8"/>
       <c r="B278" s="9"/>
       <c r="C278" s="10"/>
@@ -10016,7 +10076,7 @@
       <c r="AB278" s="13"/>
       <c r="AC278" s="13"/>
     </row>
-    <row r="279" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A279" s="8"/>
       <c r="B279" s="9"/>
       <c r="C279" s="10"/>
@@ -10046,7 +10106,7 @@
       <c r="AB279" s="13"/>
       <c r="AC279" s="13"/>
     </row>
-    <row r="280" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A280" s="8"/>
       <c r="B280" s="9"/>
       <c r="C280" s="10"/>
@@ -10076,7 +10136,7 @@
       <c r="AB280" s="13"/>
       <c r="AC280" s="13"/>
     </row>
-    <row r="281" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A281" s="8"/>
       <c r="B281" s="9"/>
       <c r="C281" s="10"/>
@@ -10106,7 +10166,7 @@
       <c r="AB281" s="13"/>
       <c r="AC281" s="13"/>
     </row>
-    <row r="282" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A282" s="8"/>
       <c r="B282" s="9"/>
       <c r="C282" s="10"/>
@@ -10136,7 +10196,7 @@
       <c r="AB282" s="13"/>
       <c r="AC282" s="13"/>
     </row>
-    <row r="283" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A283" s="8"/>
       <c r="B283" s="9"/>
       <c r="C283" s="10"/>
@@ -10166,7 +10226,7 @@
       <c r="AB283" s="13"/>
       <c r="AC283" s="13"/>
     </row>
-    <row r="284" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A284" s="8"/>
       <c r="B284" s="9"/>
       <c r="C284" s="10"/>
@@ -10196,7 +10256,7 @@
       <c r="AB284" s="13"/>
       <c r="AC284" s="13"/>
     </row>
-    <row r="285" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A285" s="8"/>
       <c r="B285" s="9"/>
       <c r="C285" s="10"/>
@@ -10226,7 +10286,7 @@
       <c r="AB285" s="13"/>
       <c r="AC285" s="13"/>
     </row>
-    <row r="286" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A286" s="8"/>
       <c r="B286" s="9"/>
       <c r="C286" s="10"/>
@@ -10256,7 +10316,7 @@
       <c r="AB286" s="13"/>
       <c r="AC286" s="13"/>
     </row>
-    <row r="287" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A287" s="8"/>
       <c r="B287" s="9"/>
       <c r="C287" s="10"/>
@@ -10286,7 +10346,7 @@
       <c r="AB287" s="13"/>
       <c r="AC287" s="13"/>
     </row>
-    <row r="288" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A288" s="8"/>
       <c r="B288" s="9"/>
       <c r="C288" s="10"/>
@@ -10316,7 +10376,7 @@
       <c r="AB288" s="13"/>
       <c r="AC288" s="13"/>
     </row>
-    <row r="289" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A289" s="8"/>
       <c r="B289" s="9"/>
       <c r="C289" s="10"/>
@@ -10346,7 +10406,7 @@
       <c r="AB289" s="13"/>
       <c r="AC289" s="13"/>
     </row>
-    <row r="290" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A290" s="8"/>
       <c r="B290" s="9"/>
       <c r="C290" s="10"/>
@@ -10376,7 +10436,7 @@
       <c r="AB290" s="13"/>
       <c r="AC290" s="13"/>
     </row>
-    <row r="291" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A291" s="8"/>
       <c r="B291" s="9"/>
       <c r="C291" s="10"/>
@@ -10406,7 +10466,7 @@
       <c r="AB291" s="13"/>
       <c r="AC291" s="13"/>
     </row>
-    <row r="292" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A292" s="8"/>
       <c r="B292" s="9"/>
       <c r="C292" s="10"/>
@@ -10436,7 +10496,7 @@
       <c r="AB292" s="13"/>
       <c r="AC292" s="13"/>
     </row>
-    <row r="293" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A293" s="8"/>
       <c r="B293" s="9"/>
       <c r="C293" s="10"/>
@@ -10466,7 +10526,7 @@
       <c r="AB293" s="13"/>
       <c r="AC293" s="13"/>
     </row>
-    <row r="294" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A294" s="8"/>
       <c r="B294" s="9"/>
       <c r="C294" s="10"/>
@@ -10496,7 +10556,7 @@
       <c r="AB294" s="13"/>
       <c r="AC294" s="13"/>
     </row>
-    <row r="295" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A295" s="8"/>
       <c r="B295" s="9"/>
       <c r="C295" s="10"/>
@@ -10526,7 +10586,7 @@
       <c r="AB295" s="13"/>
       <c r="AC295" s="13"/>
     </row>
-    <row r="296" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A296" s="8"/>
       <c r="B296" s="9"/>
       <c r="C296" s="10"/>
@@ -10556,7 +10616,7 @@
       <c r="AB296" s="13"/>
       <c r="AC296" s="13"/>
     </row>
-    <row r="297" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A297" s="8"/>
       <c r="B297" s="9"/>
       <c r="C297" s="10"/>
@@ -10586,7 +10646,7 @@
       <c r="AB297" s="13"/>
       <c r="AC297" s="13"/>
     </row>
-    <row r="298" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A298" s="8"/>
       <c r="B298" s="9"/>
       <c r="C298" s="10"/>
@@ -10616,7 +10676,7 @@
       <c r="AB298" s="13"/>
       <c r="AC298" s="13"/>
     </row>
-    <row r="299" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A299" s="8"/>
       <c r="B299" s="9"/>
       <c r="C299" s="10"/>
@@ -10646,7 +10706,7 @@
       <c r="AB299" s="13"/>
       <c r="AC299" s="13"/>
     </row>
-    <row r="300" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A300" s="8"/>
       <c r="B300" s="9"/>
       <c r="C300" s="10"/>
@@ -10676,7 +10736,7 @@
       <c r="AB300" s="13"/>
       <c r="AC300" s="13"/>
     </row>
-    <row r="301" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A301" s="8"/>
       <c r="B301" s="9"/>
       <c r="C301" s="10"/>
@@ -10706,7 +10766,7 @@
       <c r="AB301" s="13"/>
       <c r="AC301" s="13"/>
     </row>
-    <row r="302" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A302" s="8"/>
       <c r="B302" s="9"/>
       <c r="C302" s="10"/>
@@ -10736,7 +10796,7 @@
       <c r="AB302" s="13"/>
       <c r="AC302" s="13"/>
     </row>
-    <row r="303" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A303" s="8"/>
       <c r="B303" s="9"/>
       <c r="C303" s="10"/>
@@ -10766,7 +10826,7 @@
       <c r="AB303" s="13"/>
       <c r="AC303" s="13"/>
     </row>
-    <row r="304" spans="1:29" ht="13" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A304" s="8"/>
       <c r="B304" s="9"/>
       <c r="C304" s="10"/>
@@ -10874,35 +10934,36 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{217587A1-D7B2-43B1-96D2-25B9C20C0F7B}">
-  <dimension ref="A1:AM6"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A67A5FD6-9DCC-48B5-A2F2-3B411E752BAA}">
+  <dimension ref="A1:AN6"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10.6328125" customWidth="1"/>
-    <col min="3" max="3" width="14.6328125" customWidth="1"/>
-    <col min="4" max="5" width="10.6328125" customWidth="1"/>
-    <col min="6" max="6" width="14.6328125" customWidth="1"/>
-    <col min="7" max="7" width="10.6328125" customWidth="1"/>
-    <col min="8" max="8" width="11.6328125" customWidth="1"/>
-    <col min="9" max="11" width="10.6328125" customWidth="1"/>
-    <col min="12" max="12" width="30.6328125" customWidth="1"/>
-    <col min="13" max="13" width="22.6328125" customWidth="1"/>
-    <col min="14" max="16" width="10.6328125" customWidth="1"/>
-    <col min="17" max="17" width="30.6328125" customWidth="1"/>
-    <col min="18" max="18" width="26.6328125" customWidth="1"/>
-    <col min="19" max="19" width="14.6328125" customWidth="1"/>
-    <col min="20" max="20" width="30.6328125" customWidth="1"/>
-    <col min="21" max="28" width="10.6328125" customWidth="1"/>
-    <col min="29" max="29" width="24.6328125" customWidth="1"/>
-    <col min="30" max="33" width="10.6328125" customWidth="1"/>
-    <col min="34" max="34" width="50.6328125" customWidth="1"/>
-    <col min="35" max="38" width="10.6328125" customWidth="1"/>
-    <col min="39" max="39" width="20.6328125" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" customWidth="1"/>
+    <col min="4" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="12" width="10.7109375" customWidth="1"/>
+    <col min="13" max="13" width="30.7109375" customWidth="1"/>
+    <col min="14" max="14" width="22.7109375" customWidth="1"/>
+    <col min="15" max="17" width="10.7109375" customWidth="1"/>
+    <col min="18" max="18" width="30.7109375" customWidth="1"/>
+    <col min="19" max="19" width="26.7109375" customWidth="1"/>
+    <col min="20" max="20" width="14.7109375" customWidth="1"/>
+    <col min="21" max="21" width="30.7109375" customWidth="1"/>
+    <col min="22" max="29" width="10.7109375" customWidth="1"/>
+    <col min="30" max="30" width="24.7109375" customWidth="1"/>
+    <col min="31" max="34" width="10.7109375" customWidth="1"/>
+    <col min="35" max="35" width="50.7109375" customWidth="1"/>
+    <col min="36" max="39" width="10.7109375" customWidth="1"/>
+    <col min="40" max="40" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:40" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -10912,9 +10973,9 @@
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
     </row>
-    <row r="2" spans="1:39" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -10924,9 +10985,9 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:39" ht="18" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:40" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17" t="str">
@@ -10938,7 +10999,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:39" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:40" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -11056,8 +11117,11 @@
       <c r="AM5" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="6" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="AN5" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A6" t="str" cm="1">
         <f t="array" ref="A6">IF(B3="","",IFERROR(_xlfn.SORTBY(_xlfn._xlws.FILTER(Scans[],Scans[Team '#]=B3),_xlfn._xlws.FILTER(Scans[Match '#],Scans[Team '#]=B3),1),"No scans for this team yet"))</f>
         <v/>

</xml_diff>

<commit_message>
Changed to use DERT_Scouting_REBUILT.xlsx
</commit_message>
<xml_diff>
--- a/DERT_Scouting_REBUILT.xlsx
+++ b/DERT_Scouting_REBUILT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JD Projects\DERT\Scoutning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE9A8336-7E0A-4BF4-B05A-101DB48ECE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D50FF9F-8F9D-403B-9FC3-0137E684522F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{2B70F02D-221F-4FDA-B643-CA0AEB0A0C2E}"/>
+    <workbookView xWindow="29970" yWindow="1170" windowWidth="38700" windowHeight="15345" activeTab="1" xr2:uid="{0317ACFA-4569-471D-88FF-E0AB95375DE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Team Lookup" sheetId="4" r:id="rId4"/>
     <sheet name="Scouting Check" sheetId="5" r:id="rId5"/>
     <sheet name="TBA Schedule" sheetId="6" r:id="rId6"/>
+    <sheet name="TBA Teams" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,14 +38,14 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
+      <xlwcv:version warnBelowVersion="2" setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -66,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="222">
   <si>
     <t>DERT #2040 - TBA Schedule</t>
   </si>
@@ -108,6 +109,30 @@
   </si>
   <si>
     <t>Team #</t>
+  </si>
+  <si>
+    <t>DERT #2040 - TBA Teams</t>
+  </si>
+  <si>
+    <t>Paste TBA's Team List here so the Scouting Check can spot team numbers that aren't at this event, and Team Lookup can show names.</t>
+  </si>
+  <si>
+    <t>Paste the Team List here: click the yellow cell, then press Ctrl+V</t>
+  </si>
+  <si>
+    <t>HOW TO GET THE TEAM LIST</t>
+  </si>
+  <si>
+    <t>2. Under Team List, click Copy to Clipboard.</t>
+  </si>
+  <si>
+    <t>TBA usually has the team list a week or two before the event. Paste again (over the old one) if teams are added.</t>
+  </si>
+  <si>
+    <t>To remove it: select columns A to F from row 5 down and press Delete.</t>
+  </si>
+  <si>
+    <t>Name</t>
   </si>
   <si>
     <t>Schema</t>
@@ -293,7 +318,7 @@
     <t>DERT #2040 - Scouting Check</t>
   </si>
   <si>
-    <t>Problems to fix in the Scans sheet. Updates by itself; paste the TBA schedule on the TBA Schedule sheet for the full check.</t>
+    <t>Problems to fix in the Scans sheet. Updates by itself; paste TBA's team list and schedule (TBA Teams / TBA Schedule sheets) for the full check.</t>
   </si>
   <si>
     <t>Check</t>
@@ -347,6 +372,12 @@
     <t>Usually a typo in Team #: fix that cell on the Scans sheet.</t>
   </si>
   <si>
+    <t>Team not at this event</t>
+  </si>
+  <si>
+    <t>Usually a typo in Team #: fix that cell on the Scans sheet. (Checked per match instead once the schedule is pasted.)</t>
+  </si>
+  <si>
     <t>Wrong alliance</t>
   </si>
   <si>
@@ -357,6 +388,15 @@
   </si>
   <si>
     <t>See the TBA Schedule sheet.</t>
+  </si>
+  <si>
+    <t>TBA team list</t>
+  </si>
+  <si>
+    <t>See the TBA Teams sheet.</t>
+  </si>
+  <si>
+    <t>DERT #2040 - REBUILT Scouting Workbook</t>
   </si>
   <si>
     <t>Import data from the DERT Scout web app (index.html) by scanning its QR codes.</t>
@@ -395,7 +435,10 @@
     <t>CHECKING THE DATA</t>
   </si>
   <si>
-    <t>Once TBA has the match schedule (usually the day before quals), paste it on the TBA Schedule sheet - the steps are on that sheet.</t>
+    <t>Once TBA has the team list (a week or two before the event), paste it on the TBA Teams sheet. Once it has the match schedule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   (usually the day before quals), paste it on the TBA Schedule sheet. The steps are on those sheets.</t>
   </si>
   <si>
     <t>Every few matches, open the Scouting Check sheet. Red numbers = something to fix; the list below them says what and in which Excel row.</t>
@@ -422,6 +465,9 @@
     <t>TBA Schedule - paste TBA's Flat Schedule here. Nothing else to type.</t>
   </si>
   <si>
+    <t>TBA Teams - paste TBA's Team List here: catches team numbers that aren't at the event, and Team Lookup shows the team's name.</t>
+  </si>
+  <si>
     <t>LEGEND</t>
   </si>
   <si>
@@ -434,7 +480,7 @@
     <t>Ratings (Driver skill, Robot speed, Shooting accuracy) are 1 = poor to 5 = great. Multi-choice answers are separated by '; '.</t>
   </si>
   <si>
-    <t>Requires Microsoft 365 / Excel 2021 or newer (uses UNIQUE, SORTBY, FILTER, HSTACK).</t>
+    <t>Requires Microsoft 365 or Excel 2024 (uses FILTER, SORTBY, HSTACK, VSTACK, TEXTBEFORE). Excel 2021 and older show #NAME? errors.</t>
   </si>
   <si>
     <t>Schema (column A) is filled in by every QR code (S39-44228b4d for this workbook). A RED row came from a different version</t>
@@ -578,7 +624,115 @@
     <t>Submitted:  10/6/2026, 3:45:12 PM</t>
   </si>
   <si>
-    <t>DERT #2040 - REBUILT Scouting Workbook Ver 1.1</t>
+    <t>team_number,team_name,city,state_prov,country,robot_image_url</t>
+  </si>
+  <si>
+    <t>111,WildStang,Arlington Heights,Illinois,USA,https://i.imgur.com/YD2XOEam.jpg</t>
+  </si>
+  <si>
+    <t>112,Plus One,Arlington Heights,Illinois,USA,https://i.imgur.com/Npkp56Am.jpg</t>
+  </si>
+  <si>
+    <t>648,QC ELITE  Flaming Squirrels,Moline,Illinois,USA,https://i.imgur.com/wSZuD0wm.jpg</t>
+  </si>
+  <si>
+    <t>930,Mukwonago BEARs,Mukwonago,Wisconsin,USA,https://i.imgur.com/dFnSQYtm.jpg</t>
+  </si>
+  <si>
+    <t>1306,BadgerBOTS,Middleton,Wisconsin,USA,https://i.imgur.com/DfxeAa1m.jpg</t>
+  </si>
+  <si>
+    <t>1625,Winnovation,Winnebago,Illinois,USA,</t>
+  </si>
+  <si>
+    <t>1706,Ratchet Rockers,Wentzville,Missouri,USA,https://i.imgur.com/weh70Ffm.jpg</t>
+  </si>
+  <si>
+    <t>1736,Robot Casserole,Peoria,Illinois,USA,https://i.imgur.com/N1FgZ0nm.jpg</t>
+  </si>
+  <si>
+    <t>1739,Chicago Knights Robotics,Chicago,Illinois,USA,</t>
+  </si>
+  <si>
+    <t>1756,Argos,Peoria,Illinois,USA,https://i.imgur.com/WgUNKahm.jpg</t>
+  </si>
+  <si>
+    <t>1781,Lindblom Electric Eagles,Chicago,Illinois,USA,https://i.imgur.com/kB0dQZam.jpg</t>
+  </si>
+  <si>
+    <t>1792,Round Table Robotics,Oak Creek,Wisconsin,USA,https://i.imgur.com/0Hqcxc2m.jpg</t>
+  </si>
+  <si>
+    <t>2040,DERT - Dunlap Eagles Robotics Team,Dunlap,Illinois,USA,https://i.imgur.com/VLKYCJEm.jpg</t>
+  </si>
+  <si>
+    <t>2290,FLYT,Rockford,Illinois,USA,https://i.imgur.com/3Z1nhkHm.jpg</t>
+  </si>
+  <si>
+    <t>2338,Gear It Forward,Oswego,Illinois,USA,https://i.imgur.com/inmUWZPm.jpg</t>
+  </si>
+  <si>
+    <t>2481,Roboteers,Tremont,Illinois,USA,https://i.imgur.com/5ZOkuvbm.jpg</t>
+  </si>
+  <si>
+    <t>3061,Huskie Robotics,Naperville,Illinois,USA,https://i.imgur.com/4u7Fj6om.jpg</t>
+  </si>
+  <si>
+    <t>3197,HexHounds,Cedarburg,Wisconsin,USA,https://i.imgur.com/rDNJ4CWm.jpg</t>
+  </si>
+  <si>
+    <t>3397,Robolions,Saint Louis,Missouri,USA,</t>
+  </si>
+  <si>
+    <t>4096,Ctrl-Z,Champaign,Illinois,USA,https://i.imgur.com/TJWGnOAm.jpg</t>
+  </si>
+  <si>
+    <t>4143,MARS/WARS,Metamora,Illinois,USA,https://i.imgur.com/bieeiS4m.jpg</t>
+  </si>
+  <si>
+    <t>4256,Cyborg Cats,Town and Country,Missouri,USA,https://i.imgur.com/vgzMLBPm.jpg</t>
+  </si>
+  <si>
+    <t>4423,MARS' Minions,Metamora,Illinois,USA,https://i.imgur.com/MYX1Xlxm.jpg</t>
+  </si>
+  <si>
+    <t>4655,Stateline Robotics,Rockton,Illinois,USA,https://i.imgur.com/6mfDRHzm.jpg</t>
+  </si>
+  <si>
+    <t>5125,Hawks on the Horizon,Chicago,Illinois,USA,https://i.imgur.com/gBehqxSm.jpg</t>
+  </si>
+  <si>
+    <t>5822,WolfByte,Chicago,Illinois,USA,https://i.imgur.com/XebxlnWm.jpg</t>
+  </si>
+  <si>
+    <t>5847,Ironclad,Bradley,Illinois,USA,https://i.imgur.com/I5lk32bm.jpg</t>
+  </si>
+  <si>
+    <t>5934,Crowbotics,DeKalb,Illinois,USA,https://i.imgur.com/e0db8vcm.jpg</t>
+  </si>
+  <si>
+    <t>7117,Robotic Dragons,De Soto,Missouri,USA,</t>
+  </si>
+  <si>
+    <t>7457,suPURDUEper Robotics,Indianapolis,Indiana,USA,https://i.imgur.com/EdvgwX5m.jpg</t>
+  </si>
+  <si>
+    <t>9082,No Limit,Pleasant Valley,Iowa,USA,</t>
+  </si>
+  <si>
+    <t>9401,Midas' Mayhem,Troy,Missouri,USA,https://i.imgur.com/sEg4AnJm.jpg</t>
+  </si>
+  <si>
+    <t>9988,Off-Season Demo Team 9988,Manchester,NH,USA,</t>
+  </si>
+  <si>
+    <t>9996,Off-Season Demo Team 9996,Manchester,NH,USA,</t>
+  </si>
+  <si>
+    <t>9999,Off-Season Demo Team 9999,Manchester,NH,USA,</t>
+  </si>
+  <si>
+    <t>11173,STAR FORCE,Chicago,Illinois,USA,</t>
   </si>
 </sst>
 </file>
@@ -859,49 +1013,49 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6EE1F2F8-1A91-4B4A-A732-64618A828FCD}" name="Scans" displayName="Scans" ref="A1:AN2" totalsRowShown="0" headerRowDxfId="7">
-  <autoFilter ref="A1:AN2" xr:uid="{6EE1F2F8-1A91-4B4A-A732-64618A828FCD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{35B7DF69-AA67-489A-AA91-253CE54BF701}" name="Scans" displayName="Scans" ref="A1:AN2" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:AN2" xr:uid="{35B7DF69-AA67-489A-AA91-253CE54BF701}"/>
   <tableColumns count="40">
-    <tableColumn id="1" xr3:uid="{ED206498-A36E-448A-8809-E53334726048}" name="Schema"/>
-    <tableColumn id="2" xr3:uid="{74140A8F-DEE6-4EBC-A26F-8FDED34A8B4B}" name="Match type"/>
-    <tableColumn id="3" xr3:uid="{86E0B457-2A31-4C98-BF65-3E37A7D11EBD}" name="Match #"/>
-    <tableColumn id="4" xr3:uid="{6F5AC432-C732-4EFA-85DE-FC917E418D36}" name="Team #"/>
-    <tableColumn id="5" xr3:uid="{FA6F7A52-36D0-44B0-B12F-EA6B5DBC9724}" name="Alliance"/>
-    <tableColumn id="6" xr3:uid="{BFFAB8B1-2AAA-4C25-9FAF-B7490B853DD8}" name="Station"/>
-    <tableColumn id="7" xr3:uid="{10CD5623-1D01-41A0-9F3E-38D01FD1CBE0}" name="Scout name"/>
-    <tableColumn id="8" xr3:uid="{EAFEDCC9-6102-43F0-885C-C967D76E81DE}" name="Robot on field?"/>
-    <tableColumn id="9" xr3:uid="{65ABD668-01A2-4BB6-BF30-F20BBB1DB1CB}" name="Starting position"/>
-    <tableColumn id="10" xr3:uid="{37BB7C24-A390-4386-B86D-F28BDB95922E}" name="Fuel preloaded"/>
-    <tableColumn id="11" xr3:uid="{B11BC4BB-B694-43BB-B98A-A21657960D89}" name="Auto fuel scored"/>
-    <tableColumn id="12" xr3:uid="{06E3A01E-F2E3-4F2C-BAB5-1A0D5EF925D5}" name="Auto fuel missed"/>
-    <tableColumn id="13" xr3:uid="{997F1D7A-8291-438A-A0EC-32917CDEE10A}" name="Auto path"/>
-    <tableColumn id="14" xr3:uid="{AAFA7E58-D7F1-4EBB-B9BD-C031563D6654}" name="Picked up fuel from"/>
-    <tableColumn id="15" xr3:uid="{0ABD934E-2658-49B8-A7FA-2E2E914EC107}" name="Tower climb in auto"/>
-    <tableColumn id="16" xr3:uid="{1FF7890B-3030-4C17-86DE-82F3F2A53CBD}" name="Teleop fuel scored"/>
-    <tableColumn id="17" xr3:uid="{A74EEA5F-3768-411E-BADE-D6F3ADAD7E81}" name="Teleop fuel missed"/>
-    <tableColumn id="18" xr3:uid="{8F71ABEE-F2D1-4046-B0AC-AC96CF7A5A3B}" name="Intake from"/>
-    <tableColumn id="19" xr3:uid="{B0183227-4E59-4BC7-930B-675EA83C267B}" name="Shoots from"/>
-    <tableColumn id="20" xr3:uid="{C72A7FA5-7930-428F-BF59-E029F02D7B58}" name="Drives over / through"/>
-    <tableColumn id="21" xr3:uid="{26A5B46D-3374-4E62-A4CA-3A3B775C425A}" name="Inactive Hub behavior"/>
-    <tableColumn id="22" xr3:uid="{40FF2E72-0209-4CC2-84A0-05EE4D720BA8}" name="Fuel it can carry"/>
-    <tableColumn id="23" xr3:uid="{A24744D7-7413-46C5-9404-15119A12D893}" name="Played defense"/>
-    <tableColumn id="24" xr3:uid="{E512EE89-4DD1-4E69-8E02-C16BA1BD9C51}" name="Was defended"/>
-    <tableColumn id="25" xr3:uid="{9258FA73-04EC-4ACD-9AD1-9E69E1BC3CAC}" name="Tower climb"/>
-    <tableColumn id="26" xr3:uid="{31D4274C-8B48-4209-A541-3BB91FFC8C65}" name="Climb time"/>
-    <tableColumn id="27" xr3:uid="{772B5B92-9832-4EBD-81E9-3A82448D80C4}" name="Driver skill"/>
-    <tableColumn id="28" xr3:uid="{446C0323-A6C7-4C06-A401-73991AB07723}" name="Robot speed"/>
-    <tableColumn id="29" xr3:uid="{DC0C4ECE-B000-4B03-A09D-E3D69F1E7A94}" name="Shooting accuracy"/>
-    <tableColumn id="30" xr3:uid="{92A80F53-D68A-48EF-B272-9946E4E6640D}" name="Problems"/>
-    <tableColumn id="31" xr3:uid="{716A38EA-E18D-4E66-B654-B54BDD1E92E8}" name="Minor fouls"/>
-    <tableColumn id="32" xr3:uid="{B16372D3-A24C-4EC6-ACF0-39355D027803}" name="Major fouls"/>
-    <tableColumn id="33" xr3:uid="{0AB7BAD6-AC35-4FDB-8BF5-6651C6DADD9A}" name="Card"/>
-    <tableColumn id="34" xr3:uid="{3EE2911E-6E45-4677-B140-21D14CA23610}" name="Pick?"/>
-    <tableColumn id="35" xr3:uid="{FEBA64B3-830E-4B41-BABD-E10D4B19F710}" name="Observations"/>
-    <tableColumn id="36" xr3:uid="{FBF49675-4074-4059-BEC0-B035430D50A1}" name="Auto pts" dataDxfId="6"/>
-    <tableColumn id="37" xr3:uid="{DD9D6983-3714-484F-B6D3-515FB22A359E}" name="Teleop fuel pts" dataDxfId="5"/>
-    <tableColumn id="38" xr3:uid="{CA6D381F-1010-4FCB-A455-468CCB65D2B4}" name="Climb pts" dataDxfId="4"/>
-    <tableColumn id="39" xr3:uid="{A179DFED-FCDE-4526-A879-15A26E812A48}" name="Total pts" dataDxfId="3"/>
-    <tableColumn id="40" xr3:uid="{0B6CB81E-D49F-44FA-80D4-62E340A7A9D2}" name="Submitted"/>
+    <tableColumn id="1" xr3:uid="{1EA9784C-4E98-465D-B93F-D73372CA6ED9}" name="Schema"/>
+    <tableColumn id="2" xr3:uid="{F98FDB44-7263-4124-BE87-63561DCC69C4}" name="Match type"/>
+    <tableColumn id="3" xr3:uid="{6DDCE585-9FB0-4D6C-9F56-5AFA8B4CD8AA}" name="Match #"/>
+    <tableColumn id="4" xr3:uid="{8D247138-3989-4470-9D71-AD7E832A7454}" name="Team #"/>
+    <tableColumn id="5" xr3:uid="{214205A1-5EE5-4174-A32F-E31199DA3DEA}" name="Alliance"/>
+    <tableColumn id="6" xr3:uid="{1A77D063-DBAF-4FCA-97EE-44966C5FC613}" name="Station"/>
+    <tableColumn id="7" xr3:uid="{1E5796C0-77FD-4C19-8879-4C0465F88635}" name="Scout name"/>
+    <tableColumn id="8" xr3:uid="{A6A6E5F6-DA39-4074-AEB9-43AC4BEECC8E}" name="Robot on field?"/>
+    <tableColumn id="9" xr3:uid="{0A69D6E3-2B9E-4E15-8721-176E7DBAEAFD}" name="Starting position"/>
+    <tableColumn id="10" xr3:uid="{8EB6775E-A090-4B1B-A60C-0C989DE03A4C}" name="Fuel preloaded"/>
+    <tableColumn id="11" xr3:uid="{72845A38-E29A-4B09-A584-ECEB9ABBEAF1}" name="Auto fuel scored"/>
+    <tableColumn id="12" xr3:uid="{6731D0D9-190A-42BF-9D4D-B34ACB780E85}" name="Auto fuel missed"/>
+    <tableColumn id="13" xr3:uid="{EB2A6801-8BCE-4233-AA0E-13A4586A3D04}" name="Auto path"/>
+    <tableColumn id="14" xr3:uid="{56CE6720-61CF-4D1B-B4D1-4311A4AD602E}" name="Picked up fuel from"/>
+    <tableColumn id="15" xr3:uid="{E358A264-0A38-48CC-A558-E175D3E2ADCF}" name="Tower climb in auto"/>
+    <tableColumn id="16" xr3:uid="{1F21400A-4D75-499D-94F7-9FF91D9C3D0E}" name="Teleop fuel scored"/>
+    <tableColumn id="17" xr3:uid="{803ABDDD-0A49-48B5-AFE9-5ED43C34BD47}" name="Teleop fuel missed"/>
+    <tableColumn id="18" xr3:uid="{91F3ED04-8D6F-4D8C-9216-CC921714E5B2}" name="Intake from"/>
+    <tableColumn id="19" xr3:uid="{B7BF48D0-05C0-45B0-8ACD-CC4B226AFAB4}" name="Shoots from"/>
+    <tableColumn id="20" xr3:uid="{E9D24988-564E-406B-AF28-91C40FBAA9A3}" name="Drives over / through"/>
+    <tableColumn id="21" xr3:uid="{FB0BB4C7-6962-4BC8-9F8C-47193B736E50}" name="Inactive Hub behavior"/>
+    <tableColumn id="22" xr3:uid="{CCB2F81D-5938-469A-B9E2-DDBB232751CF}" name="Fuel it can carry"/>
+    <tableColumn id="23" xr3:uid="{9D601724-8D12-41DA-A037-6500714E9898}" name="Played defense"/>
+    <tableColumn id="24" xr3:uid="{D58A97B7-77ED-4648-A8B2-D565C4BAE8AB}" name="Was defended"/>
+    <tableColumn id="25" xr3:uid="{6923B0F5-C761-4706-8EDB-04D514C5395D}" name="Tower climb"/>
+    <tableColumn id="26" xr3:uid="{DA0DECF6-E0BB-4A6B-B550-CE63A8BAAE2E}" name="Climb time"/>
+    <tableColumn id="27" xr3:uid="{76A3F881-559B-4415-BB18-CE33C64216F4}" name="Driver skill"/>
+    <tableColumn id="28" xr3:uid="{BFF7C504-7FEE-475D-BAC8-84E20D4F7CA8}" name="Robot speed"/>
+    <tableColumn id="29" xr3:uid="{171247CB-DA73-4D71-B159-8FC6916F732C}" name="Shooting accuracy"/>
+    <tableColumn id="30" xr3:uid="{81504DD0-15D2-4136-ACAC-5C83935D41FD}" name="Problems"/>
+    <tableColumn id="31" xr3:uid="{8E60D869-51CF-4F11-A10A-41FA6C6654E6}" name="Minor fouls"/>
+    <tableColumn id="32" xr3:uid="{BF54C42B-4D2C-41A2-B63E-63BFB4B3A537}" name="Major fouls"/>
+    <tableColumn id="33" xr3:uid="{E9509191-90C9-4D9A-9901-8CCFCDEDD6B5}" name="Card"/>
+    <tableColumn id="34" xr3:uid="{B480B0D4-B3AF-48FC-9C92-051444184AE2}" name="Pick?"/>
+    <tableColumn id="35" xr3:uid="{5D92BC8D-3F81-49C0-9824-1D51ADCBD535}" name="Observations"/>
+    <tableColumn id="36" xr3:uid="{AA77911A-52FA-4CCF-B49C-FF6ABCD53218}" name="Auto pts" dataDxfId="6"/>
+    <tableColumn id="37" xr3:uid="{883570B7-295C-4533-B7BD-E4456BDD1FB0}" name="Teleop fuel pts" dataDxfId="5"/>
+    <tableColumn id="38" xr3:uid="{BA8F21D0-135F-410C-B4DA-FD221DC5FE2F}" name="Climb pts" dataDxfId="4"/>
+    <tableColumn id="39" xr3:uid="{C2E108E6-4364-40E6-AFE1-51F6E72C751E}" name="Total pts" dataDxfId="3"/>
+    <tableColumn id="40" xr3:uid="{FC8F8099-5900-4711-AD3F-E020FA838417}" name="Submitted"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1223,8 +1377,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5C7ADEF-4C7B-41E9-A1DE-B5F9C734F261}">
-  <dimension ref="A1:J81"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B0BA354-6ABD-4C4A-B403-BAFEC723A591}">
+  <dimension ref="A1:J83"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -1233,7 +1387,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>170</v>
+        <v>109</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1247,7 +1401,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1261,7 +1415,7 @@
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -1269,13 +1423,13 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -1283,7 +1437,7 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -1291,12 +1445,12 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -1304,7 +1458,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -1312,7 +1466,7 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1320,7 +1474,7 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -1328,12 +1482,12 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -1341,341 +1495,355 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="15">
+      <c r="A19" s="15"/>
+      <c r="B19" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="15">
         <v>2</v>
       </c>
-      <c r="B19" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="B22" t="s">
-        <v>113</v>
+      <c r="B20" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="21" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="15" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B23" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="15" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B24" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="15" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B25" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="15" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B26" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="21" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="B29" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="B30" t="s">
-        <v>120</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="B27" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="21" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="15" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B31" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="15" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="15" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" s="15"/>
+      <c r="A34" s="15" t="s">
+        <v>126</v>
+      </c>
       <c r="B34" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="B37" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="15" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="15"/>
-      <c r="B38" t="s">
-        <v>127</v>
+      <c r="B35" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="15"/>
+      <c r="B36" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="21" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" s="15"/>
+      <c r="A39" s="15" t="s">
+        <v>126</v>
+      </c>
       <c r="B39" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="21" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B42" s="22" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B43" s="22" t="s">
-        <v>131</v>
+        <v>141</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="15"/>
+      <c r="B40" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="15"/>
+      <c r="B41" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="21" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B44" s="22" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B45" s="22" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B46" s="22" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B47" s="22" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B48" s="22" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B49" s="22" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B50" s="22" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B51" s="22" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B52" s="22" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B53" s="22" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B54" s="22" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
     </row>
     <row r="55" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B55" s="22" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B56" s="22" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
     </row>
     <row r="57" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B57" s="22" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
     </row>
     <row r="58" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B58" s="22" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="59" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B59" s="22" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
     </row>
     <row r="60" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B60" s="22" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
     </row>
     <row r="61" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B61" s="22" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
     </row>
     <row r="62" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B62" s="22" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
     </row>
     <row r="63" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B63" s="22" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
     </row>
     <row r="64" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B64" s="22" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
     </row>
     <row r="65" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B65" s="22" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B66" s="22" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B67" s="22" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B68" s="22" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B69" s="22" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B70" s="22" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B71" s="22" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B72" s="22" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
     </row>
     <row r="73" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B73" s="22" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B74" s="22" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B75" s="22" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B76" s="22" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B77" s="22" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B78" s="22" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
     </row>
     <row r="79" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B79" s="22" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B80" s="22" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B81" s="22" t="s">
-        <v>169</v>
+        <v>182</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B82" s="22" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B83" s="22" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -1684,7 +1852,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20120299-04E4-4B02-B3C9-878C24610423}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC800BA0-562B-4087-B435-F871A0D7DA38}">
   <dimension ref="A1:AN1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1711,10 +1879,10 @@
   <sheetData>
     <row r="1" spans="1:40" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>11</v>
@@ -1726,113 +1894,113 @@
         <v>12</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="R1" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="S1" s="8" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="T1" s="8" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="U1" s="8" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="W1" s="8" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="X1" s="8" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="Y1" s="8" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="Z1" s="8" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="AA1" s="8" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="AB1" s="8" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="AC1" s="8" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="AD1" s="8" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="AE1" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="AF1" s="8" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="AG1" s="8" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="AH1" s="8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AI1" s="8" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="AJ1" s="8" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="AK1" s="8" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="AL1" s="8" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="AM1" s="8" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="AN1" s="8" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:AN5000">
+  <conditionalFormatting sqref="A2:AN4997">
     <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
       <formula>($A2&lt;&gt;"")*($A2&lt;&gt;"S39-44228b4d")</formula>
     </cfRule>
@@ -1845,7 +2013,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0E0C83D-DB85-4819-82AF-8B14D548A557}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AF0594B-E6FF-47DA-8BFE-572E94D24BD3}">
   <dimension ref="A1:AC304"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1856,7 +2024,7 @@
   <sheetData>
     <row r="1" spans="1:29" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1878,7 +2046,7 @@
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1900,7 +2068,7 @@
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="T3" s="5" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="30" customHeight="1" x14ac:dyDescent="0.2">
@@ -1908,85 +2076,85 @@
         <v>13</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="Q4" s="10" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="U4" s="8" t="s">
         <v>13</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="AA4" s="8" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="AB4" s="8" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="AC4" s="8" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.2">
@@ -11127,7 +11295,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CA2CB74-C901-4892-8885-DBCEB0A13C00}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D06BFD8-6836-494C-80CF-010FB6B1C7D2}">
   <dimension ref="A1:AN6"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -11156,7 +11324,7 @@
   <sheetData>
     <row r="1" spans="1:40" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -11168,7 +11336,7 @@
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -11180,7 +11348,7 @@
     </row>
     <row r="3" spans="1:40" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="19" t="str">
@@ -11191,13 +11359,17 @@
         <f>IF(B3="","",IFERROR("Rank "&amp;INDEX(_xlfn.ANCHORARRAY('Team Summary'!R5),MATCH(B3,_xlfn.ANCHORARRAY('Team Summary'!A5),0))&amp;" of "&amp;ROWS(_xlfn.ANCHORARRAY('Team Summary'!A5)),"No scans yet"))</f>
         <v/>
       </c>
+      <c r="E3" s="5" t="str" cm="1">
+        <f t="array" ref="E3">IF(B3="","",IFERROR(_xlfn.XLOOKUP(B3,INDEX(_xlfn.ANCHORARRAY('TBA Teams'!$R$5),,1),INDEX(_xlfn.ANCHORARRAY('TBA Teams'!$R$5),,2),""),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="5" spans="1:40" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>11</v>
@@ -11209,109 +11381,109 @@
         <v>12</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="Q5" s="8" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="R5" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="S5" s="8" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="T5" s="8" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="U5" s="8" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="V5" s="8" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="W5" s="8" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="X5" s="8" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="Y5" s="8" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="Z5" s="8" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="AA5" s="8" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="AB5" s="8" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="AC5" s="8" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="AD5" s="8" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="AE5" s="8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="AF5" s="8" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="AG5" s="8" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="AH5" s="8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AI5" s="8" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="AJ5" s="8" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="AK5" s="8" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="AL5" s="8" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="AM5" s="8" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="AN5" s="8" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.2">
@@ -11326,7 +11498,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F2E02B0-7B12-4953-A23D-C2CE2C60F834}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3A92049-A61E-43D9-970B-0D38A825C55C}">
   <dimension ref="A1:G3000"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -11339,7 +11511,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -11350,7 +11522,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -11361,13 +11533,13 @@
     </row>
     <row r="4" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
@@ -11376,7 +11548,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="B5" s="15">
         <f>COUNTIF(Scans[Team '#],"&lt;&gt;")</f>
@@ -11385,211 +11557,223 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B6" s="15">
-        <f>COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$15),,1),"Duplicate scan")</f>
+        <f>COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$17),,1),"Duplicate scan")</f>
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B7" s="15">
-        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,"–",COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$15),,1),"Not 6 scans"))</f>
+        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,"–",COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$17),,1),"Not 6 scans"))</f>
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B8" s="15" t="str">
-        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$15),,1),"Not scouted"),"needs schedule")</f>
+        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$17),,1),"Not scouted"),"needs schedule")</f>
         <v>needs schedule</v>
       </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="B9" s="15" t="str">
-        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$15),,1),"Team not in that match"),"needs schedule")</f>
+        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$17),,1),"Team not in that match"),"needs schedule")</f>
         <v>needs schedule</v>
       </c>
       <c r="C9" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B10" s="15" t="str">
-        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$15),,1),"Wrong alliance"),"needs schedule")</f>
-        <v>needs schedule</v>
+        <v>101</v>
+      </c>
+      <c r="B10" s="15">
+        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Teams'!$R$5),,1))&gt;0,IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,"–",COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$17),,1),"Team not at this event")),"needs team list")</f>
+        <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="B11" s="15" t="str">
+        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,COUNTIF(INDEX(_xlfn.ANCHORARRAY($A$17),,1),"Wrong alliance"),"needs schedule")</f>
+        <v>needs schedule</v>
+      </c>
+      <c r="C11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="15" t="str">
         <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))&gt;0,COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),,1))/6&amp;" qual matches","not pasted yet")</f>
         <v>not pasted yet</v>
       </c>
-      <c r="C11" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="20" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14" s="8" t="s">
+      <c r="C12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="15" t="str">
+        <f>IF(COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Teams'!$R$5),,1))&gt;0,COUNT(INDEX(_xlfn.ANCHORARRAY('TBA Teams'!$R$5),,1))&amp;" teams","not pasted yet")</f>
+        <v>36 teams</v>
+      </c>
+      <c r="C13" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C16" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D16" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" t="str" cm="1">
-        <f t="array" ref="A15">_xlfn.LET(_xlpm.ty,Scans[Match type],_xlpm.mt,Scans[Match '#],_xlpm.tm,Scans[Team '#],_xlpm.al,Scans[Alliance],_xlpm.sc,Scans[Scout name],_xlpm.rw,ROW(Scans[Team '#]),_xlpm.nT,_xlfn.SEQUENCE(ROWS(_xlpm.tm)),_xlpm.has,_xlpm.tm&lt;&gt;"",_xlpm.qual,_xlpm.has*((_xlpm.ty="Qual")+(_xlpm.ty="")),_xlpm.s,_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),_xlpm.sm,INDEX(_xlpm.s,,1),_xlpm.sa,INDEX(_xlpm.s,,2),_xlpm.st,INDEX(_xlpm.s,,3),_xlpm.nS,_xlfn.SEQUENCE(ROWS(_xlpm.sm)),_xlpm.hasSched,COUNT(_xlpm.sm)&gt;0,_xlpm.dupN,COUNTIFS(Scans[Team '#],_xlpm.tm,Scans[Match '#],_xlpm.mt,Scans[Match type],_xlpm.ty),_xlpm.dup,_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nT,"Duplicate scan"),_xlpm.mt,_xlpm.tm,_xlpm.al,_xlpm.rw,_xlpm.sc,"Scanned "&amp;_xlpm.dupN&amp;" times: delete the extra row"),_xlpm.has*(_xlpm.dupN&gt;1),""),_xlpm.qm,_xlfn.UNIQUE(_xlfn._xlws.FILTER(_xlpm.mt,_xlpm.qual,"")),_xlpm.nQ,_xlfn.SEQUENCE(ROWS(_xlpm.qm)),_xlpm.qc,COUNTIFS(Scans[Match '#],_xlpm.qm,Scans[Team '#],"&lt;&gt;",Scans[Match type],"Qual")+COUNTIFS(Scans[Match '#],_xlpm.qm,Scans[Team '#],"&lt;&gt;",Scans[Match type],""),_xlpm.cnt,IF(_xlpm.hasSched,"",_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nQ,"Not 6 scans"),_xlpm.qm,IF(_xlpm.nQ,""),IF(_xlpm.nQ,""),IF(_xlpm.nQ,""),IF(_xlpm.nQ,""),_xlpm.qc&amp;" scans in this match, expected 6"),(_xlpm.qm&lt;&gt;"")*(_xlpm.qc&lt;&gt;6),"")),_xlpm.last,MAX(_xlfn._xlws.FILTER(_xlpm.mt,_xlpm.qual,0)),_xlpm.seen,COUNTIFS(Scans[Match '#],_xlpm.sm,Scans[Team '#],_xlpm.st,Scans[Match type],"Qual")+COUNTIFS(Scans[Match '#],_xlpm.sm,Scans[Team '#],_xlpm.st,Scans[Match type],""),_xlpm.miss,IF(_xlpm.hasSched,_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nS,"Not scouted"),_xlpm.sm,_xlpm.st,_xlpm.sa,IF(_xlpm.nS,""),IF(_xlpm.nS,""),IF(_xlpm.nS,"Nobody scanned this robot: ask its scout to show the QR code again (Submitted matches)")),ISNUMBER(_xlpm.sm)*(_xlpm.sm&lt;=_xlpm.last)*(_xlpm.seen=0),""),""),_xlpm.inM,COUNTIFS(_xlpm.sm,_xlpm.mt,_xlpm.st,_xlpm.tm),_xlpm.wt,IF(_xlpm.hasSched,_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nT,"Team not in that match"),_xlpm.mt,_xlpm.tm,_xlpm.al,_xlpm.rw,_xlpm.sc,IF(COUNTIFS(_xlpm.sm,_xlpm.mt)&gt;0,"Typo in Team #? Check the schedule for this match","There is no such qual match on the TBA schedule")),_xlpm.qual*(_xlpm.inM=0),""),""),_xlpm.inA,COUNTIFS(_xlpm.sm,_xlpm.mt,_xlpm.st,_xlpm.tm,_xlpm.sa,_xlpm.al),_xlpm.wa,IF(_xlpm.hasSched,_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nT,"Wrong alliance"),_xlpm.mt,_xlpm.tm,_xlpm.al,_xlpm.rw,_xlpm.sc,"The schedule says "&amp;_xlfn.XLOOKUP(_xlpm.mt&amp;"|"&amp;_xlpm.tm,_xlpm.sm&amp;"|"&amp;_xlpm.st,_xlpm.sa,"?")),_xlpm.qual*(_xlpm.inM&gt;0)*(_xlpm.inA=0),""),""),_xlpm.all,_xlfn.VSTACK(_xlpm.dup,_xlpm.cnt,_xlpm.miss,_xlpm.wt,_xlpm.wa),IFERROR(_xlfn._xlws.FILTER(_xlpm.all,IFERROR(INDEX(_xlpm.all,,1)&lt;&gt;"",FALSE)),"✓ Nothing to fix"))</f>
+      <c r="E16" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="str" cm="1">
+        <f t="array" ref="A17">_xlfn.LET(_xlpm.ty,Scans[Match type],_xlpm.mt,Scans[Match '#],_xlpm.tm,Scans[Team '#],_xlpm.al,Scans[Alliance],_xlpm.sc,Scans[Scout name],_xlpm.rw,ROW(Scans[Team '#]),_xlpm.nT,_xlfn.SEQUENCE(ROWS(_xlpm.tm)),_xlpm.has,_xlpm.tm&lt;&gt;"",_xlpm.qual,_xlpm.has*((_xlpm.ty="Qual")+(_xlpm.ty="")),_xlpm.s,_xlfn.ANCHORARRAY('TBA Schedule'!$R$5),_xlpm.sm,INDEX(_xlpm.s,,1),_xlpm.sa,INDEX(_xlpm.s,,2),_xlpm.st,INDEX(_xlpm.s,,3),_xlpm.nS,_xlfn.SEQUENCE(ROWS(_xlpm.sm)),_xlpm.hasSched,COUNT(_xlpm.sm)&gt;0,_xlpm.dupN,COUNTIFS(Scans[Team '#],_xlpm.tm,Scans[Match '#],_xlpm.mt,Scans[Match type],_xlpm.ty),_xlpm.dup,_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nT,"Duplicate scan"),_xlpm.mt,_xlpm.tm,_xlpm.al,_xlpm.rw,_xlpm.sc,"Scanned "&amp;_xlpm.dupN&amp;" times: delete the extra row"),_xlpm.has*(_xlpm.dupN&gt;1),""),_xlpm.qm,_xlfn.UNIQUE(_xlfn._xlws.FILTER(_xlpm.mt,_xlpm.qual,"")),_xlpm.nQ,_xlfn.SEQUENCE(ROWS(_xlpm.qm)),_xlpm.qc,COUNTIFS(Scans[Match '#],_xlpm.qm,Scans[Team '#],"&lt;&gt;",Scans[Match type],"Qual")+COUNTIFS(Scans[Match '#],_xlpm.qm,Scans[Team '#],"&lt;&gt;",Scans[Match type],""),_xlpm.cnt,IF(_xlpm.hasSched,"",_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nQ,"Not 6 scans"),_xlpm.qm,IF(_xlpm.nQ,""),IF(_xlpm.nQ,""),IF(_xlpm.nQ,""),IF(_xlpm.nQ,""),_xlpm.qc&amp;" scans in this match, expected 6"),(_xlpm.qm&lt;&gt;"")*(_xlpm.qc&lt;&gt;6),"")),_xlpm.last,MAX(_xlfn._xlws.FILTER(_xlpm.mt,_xlpm.qual,0)),_xlpm.seen,COUNTIFS(Scans[Match '#],_xlpm.sm,Scans[Team '#],_xlpm.st,Scans[Match type],"Qual")+COUNTIFS(Scans[Match '#],_xlpm.sm,Scans[Team '#],_xlpm.st,Scans[Match type],""),_xlpm.miss,IF(_xlpm.hasSched,_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nS,"Not scouted"),_xlpm.sm,_xlpm.st,_xlpm.sa,IF(_xlpm.nS,""),IF(_xlpm.nS,""),IF(_xlpm.nS,"Nobody scanned this robot: ask its scout to show the QR code again (Submitted matches)")),ISNUMBER(_xlpm.sm)*(_xlpm.sm&lt;=_xlpm.last)*(_xlpm.seen=0),""),""),_xlpm.inM,COUNTIFS(_xlpm.sm,_xlpm.mt,_xlpm.st,_xlpm.tm),_xlpm.wt,IF(_xlpm.hasSched,_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nT,"Team not in that match"),_xlpm.mt,_xlpm.tm,_xlpm.al,_xlpm.rw,_xlpm.sc,IF(COUNTIFS(_xlpm.sm,_xlpm.mt)&gt;0,"Typo in Team #? Check the schedule for this match","There is no such qual match on the TBA schedule")),_xlpm.qual*(_xlpm.inM=0),""),""),_xlpm.inA,COUNTIFS(_xlpm.sm,_xlpm.mt,_xlpm.st,_xlpm.tm,_xlpm.sa,_xlpm.al),_xlpm.wa,IF(_xlpm.hasSched,_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nT,"Wrong alliance"),_xlpm.mt,_xlpm.tm,_xlpm.al,_xlpm.rw,_xlpm.sc,"The schedule says "&amp;_xlfn.XLOOKUP(_xlpm.mt&amp;"|"&amp;_xlpm.tm,_xlpm.sm&amp;"|"&amp;_xlpm.st,_xlpm.sa,"?")),_xlpm.qual*(_xlpm.inM&gt;0)*(_xlpm.inA=0),""),""),_xlpm.tl,_xlfn.ANCHORARRAY('TBA Teams'!$R$5),_xlpm.tn,INDEX(_xlpm.tl,,1),_xlpm.hasTeams,COUNT(_xlpm.tn)&gt;0,_xlpm.ne,IF(_xlpm.hasTeams*NOT(_xlpm.hasSched),_xlfn._xlws.FILTER(_xlfn.HSTACK(IF(_xlpm.nT,"Team not at this event"),_xlpm.mt,_xlpm.tm,_xlpm.al,_xlpm.rw,_xlpm.sc,IF(_xlpm.nT,"Not on TBA's team list for this event: typo in Team #?")),_xlpm.has*(COUNTIFS(_xlpm.tn,_xlpm.tm)=0),""),""),_xlpm.all,_xlfn.VSTACK(_xlpm.dup,_xlpm.cnt,_xlpm.miss,_xlpm.wt,_xlpm.ne,_xlpm.wa),_xlfn._xlws.FILTER(_xlpm.all,IFERROR(INDEX(_xlpm.all,,1)&lt;&gt;"",FALSE),"✓ Nothing to fix"))</f>
         <v>✓ Nothing to fix</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
       <c r="D19" s="15"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
       <c r="D23" s="15"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
       <c r="D26" s="15"/>
       <c r="E26" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
       <c r="D27" s="15"/>
       <c r="E27" s="15"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
       <c r="D29" s="15"/>
       <c r="E29" s="15"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
       <c r="D30" s="15"/>
       <c r="E30" s="15"/>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="15"/>
@@ -29404,7 +29588,7 @@
       <c r="E3000" s="15"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B6:B10">
+  <conditionalFormatting sqref="B6:B11">
     <cfRule type="cellIs" dxfId="1" priority="1" stopIfTrue="1" operator="between">
       <formula>1</formula>
       <formula>1E+307</formula>
@@ -29418,7 +29602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{177179F2-71CF-4F28-904C-132625E8025F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{116573B7-BDC6-49B3-AB7D-B28EE245F622}">
   <dimension ref="A1:T10"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -29541,4 +29725,502 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{032FB87A-E3D5-4673-A30E-E9B7BE200E0B}">
+  <dimension ref="A1:S41"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="62.7109375" customWidth="1"/>
+    <col min="10" max="10" width="3.7109375" customWidth="1"/>
+    <col min="18" max="18" width="10.7109375" customWidth="1"/>
+    <col min="19" max="19" width="36.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R3" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="S4" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="J5" t="s">
+        <v>4</v>
+      </c>
+      <c r="R5" cm="1">
+        <f t="array" ref="R5:S40">_xlfn.LET(_xlpm.src,A1:F1000,_xlpm.a,INDEX(_xlpm.src,,1),_xlpm.b,INDEX(_xlpm.src,,2),_xlpm.split,_xlpm.b&lt;&gt;"",_xlpm.num,IFERROR(--IF(_xlpm.split,_xlpm.a,_xlfn.TEXTBEFORE(_xlpm.a&amp;",",",")),""),_xlpm.rest,IFERROR(_xlfn.TEXTAFTER(_xlpm.a,","),""),_xlpm.name,IF(_xlpm.split,_xlpm.b,IF(LEFT(_xlpm.rest,1)="""",IFERROR(_xlfn.TEXTBEFORE(MID(_xlpm.rest,2,500),""""),""),IFERROR(_xlfn.TEXTBEFORE(_xlpm.rest&amp;",",","),""))),IFERROR(_xlfn._xlws.FILTER(_xlfn.HSTACK(_xlpm.num,_xlpm.name),ISNUMBER(_xlpm.num)),_xlfn.HSTACK("","")))</f>
+        <v>111</v>
+      </c>
+      <c r="S5" t="str">
+        <v>WildStang</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>186</v>
+      </c>
+      <c r="J6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R6">
+        <v>112</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Plus One</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>187</v>
+      </c>
+      <c r="J7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R7">
+        <v>648</v>
+      </c>
+      <c r="S7" t="str">
+        <v>QC ELITE  Flaming Squirrels</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>188</v>
+      </c>
+      <c r="J8" t="s">
+        <v>19</v>
+      </c>
+      <c r="R8">
+        <v>930</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Mukwonago BEARs</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>189</v>
+      </c>
+      <c r="J9" t="s">
+        <v>20</v>
+      </c>
+      <c r="R9">
+        <v>1306</v>
+      </c>
+      <c r="S9" t="str">
+        <v>BadgerBOTS</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>190</v>
+      </c>
+      <c r="R10">
+        <v>1625</v>
+      </c>
+      <c r="S10" t="str">
+        <v>Winnovation</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>191</v>
+      </c>
+      <c r="R11">
+        <v>1706</v>
+      </c>
+      <c r="S11" t="str">
+        <v>Ratchet Rockers</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>192</v>
+      </c>
+      <c r="R12">
+        <v>1736</v>
+      </c>
+      <c r="S12" t="str">
+        <v>Robot Casserole</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>193</v>
+      </c>
+      <c r="R13">
+        <v>1739</v>
+      </c>
+      <c r="S13" t="str">
+        <v>Chicago Knights Robotics</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>194</v>
+      </c>
+      <c r="R14">
+        <v>1756</v>
+      </c>
+      <c r="S14" t="str">
+        <v>Argos</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>195</v>
+      </c>
+      <c r="R15">
+        <v>1781</v>
+      </c>
+      <c r="S15" t="str">
+        <v>Lindblom Electric Eagles</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>196</v>
+      </c>
+      <c r="R16">
+        <v>1792</v>
+      </c>
+      <c r="S16" t="str">
+        <v>Round Table Robotics</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>197</v>
+      </c>
+      <c r="R17">
+        <v>2040</v>
+      </c>
+      <c r="S17" t="str">
+        <v>DERT - Dunlap Eagles Robotics Team</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>198</v>
+      </c>
+      <c r="R18">
+        <v>2290</v>
+      </c>
+      <c r="S18" t="str">
+        <v>FLYT</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>199</v>
+      </c>
+      <c r="R19">
+        <v>2338</v>
+      </c>
+      <c r="S19" t="str">
+        <v>Gear It Forward</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>200</v>
+      </c>
+      <c r="R20">
+        <v>2481</v>
+      </c>
+      <c r="S20" t="str">
+        <v>Roboteers</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>201</v>
+      </c>
+      <c r="R21">
+        <v>3061</v>
+      </c>
+      <c r="S21" t="str">
+        <v>Huskie Robotics</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>202</v>
+      </c>
+      <c r="R22">
+        <v>3197</v>
+      </c>
+      <c r="S22" t="str">
+        <v>HexHounds</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>203</v>
+      </c>
+      <c r="R23">
+        <v>3397</v>
+      </c>
+      <c r="S23" t="str">
+        <v>Robolions</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>204</v>
+      </c>
+      <c r="R24">
+        <v>4096</v>
+      </c>
+      <c r="S24" t="str">
+        <v>Ctrl-Z</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>205</v>
+      </c>
+      <c r="R25">
+        <v>4143</v>
+      </c>
+      <c r="S25" t="str">
+        <v>MARS/WARS</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>206</v>
+      </c>
+      <c r="R26">
+        <v>4256</v>
+      </c>
+      <c r="S26" t="str">
+        <v>Cyborg Cats</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>207</v>
+      </c>
+      <c r="R27">
+        <v>4423</v>
+      </c>
+      <c r="S27" t="str">
+        <v>MARS' Minions</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>208</v>
+      </c>
+      <c r="R28">
+        <v>4655</v>
+      </c>
+      <c r="S28" t="str">
+        <v>Stateline Robotics</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>209</v>
+      </c>
+      <c r="R29">
+        <v>5125</v>
+      </c>
+      <c r="S29" t="str">
+        <v>Hawks on the Horizon</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>210</v>
+      </c>
+      <c r="R30">
+        <v>5822</v>
+      </c>
+      <c r="S30" t="str">
+        <v>WolfByte</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>211</v>
+      </c>
+      <c r="R31">
+        <v>5847</v>
+      </c>
+      <c r="S31" t="str">
+        <v>Ironclad</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>212</v>
+      </c>
+      <c r="R32">
+        <v>5934</v>
+      </c>
+      <c r="S32" t="str">
+        <v>Crowbotics</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>213</v>
+      </c>
+      <c r="R33">
+        <v>7117</v>
+      </c>
+      <c r="S33" t="str">
+        <v>Robotic Dragons</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>214</v>
+      </c>
+      <c r="R34">
+        <v>7457</v>
+      </c>
+      <c r="S34" t="str">
+        <v>suPURDUEper Robotics</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>215</v>
+      </c>
+      <c r="R35">
+        <v>9082</v>
+      </c>
+      <c r="S35" t="str">
+        <v>No Limit</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>216</v>
+      </c>
+      <c r="R36">
+        <v>9401</v>
+      </c>
+      <c r="S36" t="str">
+        <v>Midas' Mayhem</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>217</v>
+      </c>
+      <c r="R37">
+        <v>9988</v>
+      </c>
+      <c r="S37" t="str">
+        <v>Off-Season Demo Team 9988</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>218</v>
+      </c>
+      <c r="R38">
+        <v>9996</v>
+      </c>
+      <c r="S38" t="str">
+        <v>Off-Season Demo Team 9996</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>219</v>
+      </c>
+      <c r="R39">
+        <v>9999</v>
+      </c>
+      <c r="S39" t="str">
+        <v>Off-Season Demo Team 9999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>220</v>
+      </c>
+      <c r="R40">
+        <v>11173</v>
+      </c>
+      <c r="S40" t="str">
+        <v>STAR FORCE</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>221</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>